<commit_message>
fix: add metadata sheet
</commit_message>
<xml_diff>
--- a/xlsx/tests/templates/event_calendar.xlsx
+++ b/xlsx/tests/templates/event_calendar.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dg-ac/Documents/IronCalc Mkt/Templates/final/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E737AF3D-1BEB-0F4B-BDD6-69ED0365DACE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADFA7017-D500-2946-8ED7-52ABB6E6E4CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3980" yWindow="-19400" windowWidth="33960" windowHeight="17260" xr2:uid="{6F0581DF-A6A1-8847-8CD1-D7A1DAEC65B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Event calendar" sheetId="1" r:id="rId1"/>
+    <sheet name="METADATA" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -61,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="9">
   <si>
     <t>D</t>
   </si>
@@ -85,6 +86,9 @@
   </si>
   <si>
     <t>Isaac Newton's birthday</t>
+  </si>
+  <si>
+    <t>NOW</t>
   </si>
 </sst>
 </file>
@@ -238,7 +242,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -305,6 +309,7 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8754,4 +8759,26 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A79E5012-AEC7-9F43-B1A8-1E796EAAC6CB}">
+  <dimension ref="A2:B2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="24">
+        <f ca="1">NOW()</f>
+        <v>46226.526188541669</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: WEEK() formula in events calendar
</commit_message>
<xml_diff>
--- a/xlsx/tests/templates/event_calendar.xlsx
+++ b/xlsx/tests/templates/event_calendar.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dg-ac/Documents/IronCalc Mkt/Templates/final/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dg-ac/Documents/IronCalc/xlsx/tests/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADFA7017-D500-2946-8ED7-52ABB6E6E4CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C97CE2C-3D87-5E44-A011-2B62E069B4B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3980" yWindow="-19400" windowWidth="33960" windowHeight="17260" xr2:uid="{6F0581DF-A6A1-8847-8CD1-D7A1DAEC65B8}"/>
   </bookViews>
@@ -16,6 +16,9 @@
     <sheet name="Event calendar" sheetId="1" r:id="rId1"/>
     <sheet name="METADATA" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="week">_xlfn.LAMBDA(LEFT(TEXT(2+_xlfn.SEQUENCE(1,7,0),"ddd")))</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -40,7 +43,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -1350,351 +1353,279 @@
     </row>
     <row r="5" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1"/>
-      <c r="B5" s="2" t="str">
-        <f>LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($B$5),"dddd"),1)</f>
+      <c r="B5" s="2" t="str" cm="1">
+        <f t="array" ref="B5:H5">week()</f>
         <v>M</v>
       </c>
       <c r="C5" s="2" t="str">
-        <f t="shared" ref="C5:H5" si="0">LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($B$5),"dddd"),1)</f>
         <v>T</v>
       </c>
       <c r="D5" s="2" t="str">
-        <f t="shared" si="0"/>
         <v>W</v>
       </c>
       <c r="E5" s="2" t="str">
-        <f t="shared" si="0"/>
         <v>T</v>
       </c>
       <c r="F5" s="2" t="str">
-        <f t="shared" si="0"/>
         <v>F</v>
       </c>
       <c r="G5" s="23" t="str">
-        <f t="shared" si="0"/>
         <v>S</v>
       </c>
       <c r="H5" s="23" t="str">
-        <f t="shared" si="0"/>
         <v>S</v>
       </c>
       <c r="I5" s="19"/>
-      <c r="J5" s="2" t="str">
-        <f>LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($J$5),"dddd"),1)</f>
+      <c r="J5" s="2" t="str" cm="1">
+        <f t="array" ref="J5:P5">week()</f>
         <v>M</v>
       </c>
       <c r="K5" s="2" t="str">
-        <f t="shared" ref="K5:P5" si="1">LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($J$5),"dddd"),1)</f>
         <v>T</v>
       </c>
       <c r="L5" s="2" t="str">
-        <f t="shared" si="1"/>
         <v>W</v>
       </c>
       <c r="M5" s="2" t="str">
-        <f t="shared" si="1"/>
         <v>T</v>
       </c>
       <c r="N5" s="2" t="str">
-        <f t="shared" si="1"/>
         <v>F</v>
       </c>
       <c r="O5" s="23" t="str">
-        <f t="shared" si="1"/>
         <v>S</v>
       </c>
       <c r="P5" s="23" t="str">
-        <f t="shared" si="1"/>
         <v>S</v>
       </c>
       <c r="Q5" s="19"/>
-      <c r="R5" s="2" t="str">
-        <f t="shared" ref="R5:X5" si="2">LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($R$5),"dddd"),1)</f>
+      <c r="R5" s="2" t="str" cm="1">
+        <f t="array" ref="R5:X5">week()</f>
         <v>M</v>
       </c>
       <c r="S5" s="2" t="str">
-        <f t="shared" si="2"/>
         <v>T</v>
       </c>
       <c r="T5" s="2" t="str">
-        <f t="shared" si="2"/>
         <v>W</v>
       </c>
       <c r="U5" s="2" t="str">
-        <f t="shared" si="2"/>
         <v>T</v>
       </c>
       <c r="V5" s="2" t="str">
-        <f t="shared" si="2"/>
         <v>F</v>
       </c>
       <c r="W5" s="23" t="str">
-        <f t="shared" si="2"/>
         <v>S</v>
       </c>
       <c r="X5" s="23" t="str">
-        <f t="shared" si="2"/>
         <v>S</v>
       </c>
       <c r="Y5" s="19"/>
-      <c r="Z5" s="2" t="str">
-        <f t="shared" ref="Z5:AF5" si="3">LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($Z$5),"dddd"),1)</f>
+      <c r="Z5" s="2" t="str" cm="1">
+        <f t="array" ref="Z5:AF5">week()</f>
         <v>M</v>
       </c>
       <c r="AA5" s="2" t="str">
-        <f t="shared" si="3"/>
         <v>T</v>
       </c>
       <c r="AB5" s="2" t="str">
-        <f t="shared" si="3"/>
         <v>W</v>
       </c>
       <c r="AC5" s="2" t="str">
-        <f t="shared" si="3"/>
         <v>T</v>
       </c>
       <c r="AD5" s="2" t="str">
-        <f t="shared" si="3"/>
         <v>F</v>
       </c>
       <c r="AE5" s="23" t="str">
-        <f t="shared" si="3"/>
         <v>S</v>
       </c>
       <c r="AF5" s="23" t="str">
-        <f t="shared" si="3"/>
         <v>S</v>
       </c>
       <c r="AG5" s="19"/>
-      <c r="AH5" s="2" t="str">
-        <f t="shared" ref="AH5:AN5" si="4">LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($AH$5),"dddd"),1)</f>
+      <c r="AH5" s="2" t="str" cm="1">
+        <f t="array" ref="AH5:AN5">week()</f>
         <v>M</v>
       </c>
       <c r="AI5" s="2" t="str">
-        <f t="shared" si="4"/>
         <v>T</v>
       </c>
       <c r="AJ5" s="2" t="str">
-        <f t="shared" si="4"/>
         <v>W</v>
       </c>
       <c r="AK5" s="2" t="str">
-        <f t="shared" si="4"/>
         <v>T</v>
       </c>
       <c r="AL5" s="2" t="str">
-        <f t="shared" si="4"/>
         <v>F</v>
       </c>
       <c r="AM5" s="23" t="str">
-        <f t="shared" si="4"/>
         <v>S</v>
       </c>
       <c r="AN5" s="23" t="str">
-        <f t="shared" si="4"/>
         <v>S</v>
       </c>
       <c r="AO5" s="19"/>
-      <c r="AP5" s="2" t="str">
-        <f t="shared" ref="AP5:AV5" si="5">LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($AP$5),"dddd"),1)</f>
+      <c r="AP5" s="2" t="str" cm="1">
+        <f t="array" ref="AP5:AV5">week()</f>
         <v>M</v>
       </c>
       <c r="AQ5" s="2" t="str">
-        <f t="shared" si="5"/>
         <v>T</v>
       </c>
       <c r="AR5" s="2" t="str">
-        <f t="shared" si="5"/>
         <v>W</v>
       </c>
       <c r="AS5" s="2" t="str">
-        <f t="shared" si="5"/>
         <v>T</v>
       </c>
       <c r="AT5" s="2" t="str">
-        <f t="shared" si="5"/>
         <v>F</v>
       </c>
       <c r="AU5" s="23" t="str">
-        <f t="shared" si="5"/>
         <v>S</v>
       </c>
       <c r="AV5" s="23" t="str">
-        <f t="shared" si="5"/>
         <v>S</v>
       </c>
       <c r="AW5" s="19"/>
-      <c r="AX5" s="2" t="str">
-        <f t="shared" ref="AX5:BD5" si="6">LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($AX$5),"dddd"),1)</f>
+      <c r="AX5" s="2" t="str" cm="1">
+        <f t="array" ref="AX5:BD5">week()</f>
         <v>M</v>
       </c>
       <c r="AY5" s="2" t="str">
-        <f t="shared" si="6"/>
         <v>T</v>
       </c>
       <c r="AZ5" s="2" t="str">
-        <f t="shared" si="6"/>
         <v>W</v>
       </c>
       <c r="BA5" s="2" t="str">
-        <f t="shared" si="6"/>
         <v>T</v>
       </c>
       <c r="BB5" s="2" t="str">
-        <f t="shared" si="6"/>
         <v>F</v>
       </c>
       <c r="BC5" s="23" t="str">
-        <f t="shared" si="6"/>
         <v>S</v>
       </c>
       <c r="BD5" s="23" t="str">
-        <f t="shared" si="6"/>
         <v>S</v>
       </c>
       <c r="BE5" s="19"/>
-      <c r="BF5" s="2" t="str">
-        <f t="shared" ref="BF5:BL5" si="7">LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($BF$5),"dddd"),1)</f>
+      <c r="BF5" s="2" t="str" cm="1">
+        <f t="array" ref="BF5:BL5">week()</f>
         <v>M</v>
       </c>
       <c r="BG5" s="2" t="str">
-        <f t="shared" si="7"/>
         <v>T</v>
       </c>
       <c r="BH5" s="2" t="str">
-        <f t="shared" si="7"/>
         <v>W</v>
       </c>
       <c r="BI5" s="2" t="str">
-        <f t="shared" si="7"/>
         <v>T</v>
       </c>
       <c r="BJ5" s="2" t="str">
-        <f t="shared" si="7"/>
         <v>F</v>
       </c>
       <c r="BK5" s="23" t="str">
-        <f t="shared" si="7"/>
         <v>S</v>
       </c>
       <c r="BL5" s="23" t="str">
-        <f t="shared" si="7"/>
         <v>S</v>
       </c>
       <c r="BM5" s="19"/>
-      <c r="BN5" s="2" t="str">
-        <f t="shared" ref="BN5:BT5" si="8">LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($BN$5),"dddd"),1)</f>
+      <c r="BN5" s="2" t="str" cm="1">
+        <f t="array" ref="BN5:BT5">week()</f>
         <v>M</v>
       </c>
       <c r="BO5" s="2" t="str">
-        <f t="shared" si="8"/>
         <v>T</v>
       </c>
       <c r="BP5" s="2" t="str">
-        <f t="shared" si="8"/>
         <v>W</v>
       </c>
       <c r="BQ5" s="2" t="str">
-        <f t="shared" si="8"/>
         <v>T</v>
       </c>
       <c r="BR5" s="2" t="str">
-        <f t="shared" si="8"/>
         <v>F</v>
       </c>
       <c r="BS5" s="23" t="str">
-        <f t="shared" si="8"/>
         <v>S</v>
       </c>
       <c r="BT5" s="23" t="str">
-        <f t="shared" si="8"/>
         <v>S</v>
       </c>
       <c r="BU5" s="19"/>
-      <c r="BV5" s="2" t="str">
-        <f t="shared" ref="BV5:CB5" si="9">LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($BV$5),"dddd"),1)</f>
+      <c r="BV5" s="2" t="str" cm="1">
+        <f t="array" ref="BV5:CB5">week()</f>
         <v>M</v>
       </c>
       <c r="BW5" s="2" t="str">
-        <f t="shared" si="9"/>
         <v>T</v>
       </c>
       <c r="BX5" s="2" t="str">
-        <f t="shared" si="9"/>
         <v>W</v>
       </c>
       <c r="BY5" s="2" t="str">
-        <f t="shared" si="9"/>
         <v>T</v>
       </c>
       <c r="BZ5" s="2" t="str">
-        <f t="shared" si="9"/>
         <v>F</v>
       </c>
       <c r="CA5" s="23" t="str">
-        <f t="shared" si="9"/>
         <v>S</v>
       </c>
       <c r="CB5" s="23" t="str">
-        <f t="shared" si="9"/>
         <v>S</v>
       </c>
       <c r="CC5" s="19"/>
-      <c r="CD5" s="2" t="str">
-        <f t="shared" ref="CD5:CJ5" si="10">LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($CD$5),"dddd"),1)</f>
+      <c r="CD5" s="2" t="str" cm="1">
+        <f t="array" ref="CD5:CJ5">week()</f>
         <v>M</v>
       </c>
       <c r="CE5" s="2" t="str">
-        <f t="shared" si="10"/>
         <v>T</v>
       </c>
       <c r="CF5" s="2" t="str">
-        <f t="shared" si="10"/>
         <v>W</v>
       </c>
       <c r="CG5" s="2" t="str">
-        <f t="shared" si="10"/>
         <v>T</v>
       </c>
       <c r="CH5" s="2" t="str">
-        <f t="shared" si="10"/>
         <v>F</v>
       </c>
       <c r="CI5" s="23" t="str">
-        <f t="shared" si="10"/>
         <v>S</v>
       </c>
       <c r="CJ5" s="23" t="str">
-        <f t="shared" si="10"/>
         <v>S</v>
       </c>
       <c r="CK5" s="19"/>
-      <c r="CL5" s="2" t="str">
-        <f t="shared" ref="CL5:CR5" si="11">LEFT(TEXT(DATE(2024,1,1)+COLUMN()-COLUMN($CL$5),"dddd"),1)</f>
+      <c r="CL5" s="2" t="str" cm="1">
+        <f t="array" ref="CL5:CR5">week()</f>
         <v>M</v>
       </c>
       <c r="CM5" s="2" t="str">
-        <f t="shared" si="11"/>
         <v>T</v>
       </c>
       <c r="CN5" s="2" t="str">
-        <f t="shared" si="11"/>
         <v>W</v>
       </c>
       <c r="CO5" s="2" t="str">
-        <f t="shared" si="11"/>
         <v>T</v>
       </c>
       <c r="CP5" s="2" t="str">
-        <f t="shared" si="11"/>
         <v>F</v>
       </c>
       <c r="CQ5" s="23" t="str">
-        <f t="shared" si="11"/>
         <v>S</v>
       </c>
       <c r="CR5" s="23" t="str">
-        <f t="shared" si="11"/>
         <v>S</v>
       </c>
       <c r="CS5" s="15"/>
@@ -4346,7 +4277,7 @@
       <c r="P16" s="21"/>
       <c r="Q16" s="19"/>
       <c r="R16" s="13">
-        <f t="shared" ref="R16:R45" ca="1" si="12">R15+1</f>
+        <f t="shared" ref="R16:R45" ca="1" si="0">R15+1</f>
         <v>46083</v>
       </c>
       <c r="S16" s="12"/>
@@ -4357,7 +4288,7 @@
       <c r="X16" s="21"/>
       <c r="Y16" s="19"/>
       <c r="Z16" s="13">
-        <f t="shared" ref="Z16:Z44" ca="1" si="13">Z15+1</f>
+        <f t="shared" ref="Z16:Z44" ca="1" si="1">Z15+1</f>
         <v>46114</v>
       </c>
       <c r="AA16" s="12"/>
@@ -4368,7 +4299,7 @@
       <c r="AF16" s="21"/>
       <c r="AG16" s="19"/>
       <c r="AH16" s="13">
-        <f t="shared" ref="AH16:AH45" ca="1" si="14">AH15+1</f>
+        <f t="shared" ref="AH16:AH45" ca="1" si="2">AH15+1</f>
         <v>46144</v>
       </c>
       <c r="AI16" s="12"/>
@@ -4379,7 +4310,7 @@
       <c r="AN16" s="21"/>
       <c r="AO16" s="19"/>
       <c r="AP16" s="13">
-        <f t="shared" ref="AP16:AP44" ca="1" si="15">AP15+1</f>
+        <f t="shared" ref="AP16:AP44" ca="1" si="3">AP15+1</f>
         <v>46175</v>
       </c>
       <c r="AQ16" s="12"/>
@@ -4390,7 +4321,7 @@
       <c r="AV16" s="21"/>
       <c r="AW16" s="19"/>
       <c r="AX16" s="13">
-        <f t="shared" ref="AX16:AX45" ca="1" si="16">AX15+1</f>
+        <f t="shared" ref="AX16:AX45" ca="1" si="4">AX15+1</f>
         <v>46205</v>
       </c>
       <c r="AY16" s="12"/>
@@ -4401,7 +4332,7 @@
       <c r="BD16" s="21"/>
       <c r="BE16" s="19"/>
       <c r="BF16" s="13">
-        <f t="shared" ref="BF16:BF45" ca="1" si="17">BF15+1</f>
+        <f t="shared" ref="BF16:BF45" ca="1" si="5">BF15+1</f>
         <v>46236</v>
       </c>
       <c r="BG16" s="12"/>
@@ -4412,7 +4343,7 @@
       <c r="BL16" s="21"/>
       <c r="BM16" s="19"/>
       <c r="BN16" s="13">
-        <f t="shared" ref="BN16:BN44" ca="1" si="18">BN15+1</f>
+        <f t="shared" ref="BN16:BN44" ca="1" si="6">BN15+1</f>
         <v>46267</v>
       </c>
       <c r="BO16" s="12"/>
@@ -4423,7 +4354,7 @@
       <c r="BT16" s="21"/>
       <c r="BU16" s="19"/>
       <c r="BV16" s="13">
-        <f t="shared" ref="BV16:BV45" ca="1" si="19">BV15+1</f>
+        <f t="shared" ref="BV16:BV45" ca="1" si="7">BV15+1</f>
         <v>46297</v>
       </c>
       <c r="BW16" s="12"/>
@@ -4434,7 +4365,7 @@
       <c r="CB16" s="21"/>
       <c r="CC16" s="19"/>
       <c r="CD16" s="13">
-        <f t="shared" ref="CD16:CD44" ca="1" si="20">CD15+1</f>
+        <f t="shared" ref="CD16:CD44" ca="1" si="8">CD15+1</f>
         <v>46328</v>
       </c>
       <c r="CE16" s="12"/>
@@ -4445,7 +4376,7 @@
       <c r="CJ16" s="21"/>
       <c r="CK16" s="19"/>
       <c r="CL16" s="13">
-        <f t="shared" ref="CL16:CL45" ca="1" si="21">CL15+1</f>
+        <f t="shared" ref="CL16:CL45" ca="1" si="9">CL15+1</f>
         <v>46358</v>
       </c>
       <c r="CM16" s="12"/>
@@ -4459,7 +4390,7 @@
     <row r="17" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
       <c r="B17" s="13">
-        <f t="shared" ref="B17:B21" ca="1" si="22">B16+1</f>
+        <f t="shared" ref="B17:B21" ca="1" si="10">B16+1</f>
         <v>46025</v>
       </c>
       <c r="C17" s="12"/>
@@ -4470,7 +4401,7 @@
       <c r="H17" s="21"/>
       <c r="I17" s="19"/>
       <c r="J17" s="13">
-        <f t="shared" ref="J17:J42" ca="1" si="23">J16+1</f>
+        <f t="shared" ref="J17:J42" ca="1" si="11">J16+1</f>
         <v>46056</v>
       </c>
       <c r="K17" s="12"/>
@@ -4481,7 +4412,7 @@
       <c r="P17" s="21"/>
       <c r="Q17" s="19"/>
       <c r="R17" s="13">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="0"/>
         <v>46084</v>
       </c>
       <c r="S17" s="12"/>
@@ -4492,7 +4423,7 @@
       <c r="X17" s="21"/>
       <c r="Y17" s="19"/>
       <c r="Z17" s="13">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" ca="1" si="1"/>
         <v>46115</v>
       </c>
       <c r="AA17" s="12" t="s">
@@ -4505,7 +4436,7 @@
       <c r="AF17" s="21"/>
       <c r="AG17" s="19"/>
       <c r="AH17" s="13">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" ca="1" si="2"/>
         <v>46145</v>
       </c>
       <c r="AI17" s="12"/>
@@ -4516,7 +4447,7 @@
       <c r="AN17" s="21"/>
       <c r="AO17" s="19"/>
       <c r="AP17" s="13">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="3"/>
         <v>46176</v>
       </c>
       <c r="AQ17" s="12"/>
@@ -4527,7 +4458,7 @@
       <c r="AV17" s="21"/>
       <c r="AW17" s="19"/>
       <c r="AX17" s="13">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="4"/>
         <v>46206</v>
       </c>
       <c r="AY17" s="12"/>
@@ -4538,7 +4469,7 @@
       <c r="BD17" s="21"/>
       <c r="BE17" s="19"/>
       <c r="BF17" s="13">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" ca="1" si="5"/>
         <v>46237</v>
       </c>
       <c r="BG17" s="12"/>
@@ -4549,7 +4480,7 @@
       <c r="BL17" s="21"/>
       <c r="BM17" s="19"/>
       <c r="BN17" s="13">
-        <f t="shared" ca="1" si="18"/>
+        <f t="shared" ca="1" si="6"/>
         <v>46268</v>
       </c>
       <c r="BO17" s="12"/>
@@ -4560,7 +4491,7 @@
       <c r="BT17" s="21"/>
       <c r="BU17" s="19"/>
       <c r="BV17" s="13">
-        <f t="shared" ca="1" si="19"/>
+        <f t="shared" ca="1" si="7"/>
         <v>46298</v>
       </c>
       <c r="BW17" s="12"/>
@@ -4571,7 +4502,7 @@
       <c r="CB17" s="21"/>
       <c r="CC17" s="19"/>
       <c r="CD17" s="13">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" ca="1" si="8"/>
         <v>46329</v>
       </c>
       <c r="CE17" s="12"/>
@@ -4582,7 +4513,7 @@
       <c r="CJ17" s="21"/>
       <c r="CK17" s="19"/>
       <c r="CL17" s="13">
-        <f t="shared" ca="1" si="21"/>
+        <f t="shared" ca="1" si="9"/>
         <v>46359</v>
       </c>
       <c r="CM17" s="12"/>
@@ -4596,7 +4527,7 @@
     <row r="18" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
       <c r="B18" s="13">
-        <f t="shared" ca="1" si="22"/>
+        <f t="shared" ca="1" si="10"/>
         <v>46026</v>
       </c>
       <c r="C18" s="12" t="s">
@@ -4609,7 +4540,7 @@
       <c r="H18" s="21"/>
       <c r="I18" s="19"/>
       <c r="J18" s="13">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" ca="1" si="11"/>
         <v>46057</v>
       </c>
       <c r="K18" s="12"/>
@@ -4620,7 +4551,7 @@
       <c r="P18" s="21"/>
       <c r="Q18" s="19"/>
       <c r="R18" s="13">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="0"/>
         <v>46085</v>
       </c>
       <c r="S18" s="12"/>
@@ -4631,7 +4562,7 @@
       <c r="X18" s="21"/>
       <c r="Y18" s="19"/>
       <c r="Z18" s="13">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" ca="1" si="1"/>
         <v>46116</v>
       </c>
       <c r="AA18" s="12"/>
@@ -4642,7 +4573,7 @@
       <c r="AF18" s="21"/>
       <c r="AG18" s="19"/>
       <c r="AH18" s="13">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" ca="1" si="2"/>
         <v>46146</v>
       </c>
       <c r="AI18" s="12"/>
@@ -4653,7 +4584,7 @@
       <c r="AN18" s="21"/>
       <c r="AO18" s="19"/>
       <c r="AP18" s="13">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="3"/>
         <v>46177</v>
       </c>
       <c r="AQ18" s="12"/>
@@ -4664,7 +4595,7 @@
       <c r="AV18" s="21"/>
       <c r="AW18" s="19"/>
       <c r="AX18" s="13">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="4"/>
         <v>46207</v>
       </c>
       <c r="AY18" s="12"/>
@@ -4675,7 +4606,7 @@
       <c r="BD18" s="21"/>
       <c r="BE18" s="19"/>
       <c r="BF18" s="13">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" ca="1" si="5"/>
         <v>46238</v>
       </c>
       <c r="BG18" s="12"/>
@@ -4686,7 +4617,7 @@
       <c r="BL18" s="21"/>
       <c r="BM18" s="19"/>
       <c r="BN18" s="13">
-        <f t="shared" ca="1" si="18"/>
+        <f t="shared" ca="1" si="6"/>
         <v>46269</v>
       </c>
       <c r="BO18" s="12"/>
@@ -4697,7 +4628,7 @@
       <c r="BT18" s="21"/>
       <c r="BU18" s="19"/>
       <c r="BV18" s="13">
-        <f t="shared" ca="1" si="19"/>
+        <f t="shared" ca="1" si="7"/>
         <v>46299</v>
       </c>
       <c r="BW18" s="12"/>
@@ -4708,7 +4639,7 @@
       <c r="CB18" s="21"/>
       <c r="CC18" s="19"/>
       <c r="CD18" s="13">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" ca="1" si="8"/>
         <v>46330</v>
       </c>
       <c r="CE18" s="12"/>
@@ -4719,7 +4650,7 @@
       <c r="CJ18" s="21"/>
       <c r="CK18" s="19"/>
       <c r="CL18" s="13">
-        <f t="shared" ca="1" si="21"/>
+        <f t="shared" ca="1" si="9"/>
         <v>46360</v>
       </c>
       <c r="CM18" s="12"/>
@@ -4733,7 +4664,7 @@
     <row r="19" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1"/>
       <c r="B19" s="13">
-        <f t="shared" ca="1" si="22"/>
+        <f t="shared" ca="1" si="10"/>
         <v>46027</v>
       </c>
       <c r="C19" s="12"/>
@@ -4744,7 +4675,7 @@
       <c r="H19" s="21"/>
       <c r="I19" s="19"/>
       <c r="J19" s="13">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" ca="1" si="11"/>
         <v>46058</v>
       </c>
       <c r="K19" s="12"/>
@@ -4755,7 +4686,7 @@
       <c r="P19" s="21"/>
       <c r="Q19" s="19"/>
       <c r="R19" s="13">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="0"/>
         <v>46086</v>
       </c>
       <c r="S19" s="12"/>
@@ -4766,7 +4697,7 @@
       <c r="X19" s="21"/>
       <c r="Y19" s="19"/>
       <c r="Z19" s="13">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" ca="1" si="1"/>
         <v>46117</v>
       </c>
       <c r="AA19" s="12"/>
@@ -4777,7 +4708,7 @@
       <c r="AF19" s="21"/>
       <c r="AG19" s="19"/>
       <c r="AH19" s="13">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" ca="1" si="2"/>
         <v>46147</v>
       </c>
       <c r="AI19" s="12"/>
@@ -4788,7 +4719,7 @@
       <c r="AN19" s="21"/>
       <c r="AO19" s="19"/>
       <c r="AP19" s="13">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="3"/>
         <v>46178</v>
       </c>
       <c r="AQ19" s="12"/>
@@ -4799,7 +4730,7 @@
       <c r="AV19" s="21"/>
       <c r="AW19" s="19"/>
       <c r="AX19" s="13">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="4"/>
         <v>46208</v>
       </c>
       <c r="AY19" s="12"/>
@@ -4810,7 +4741,7 @@
       <c r="BD19" s="21"/>
       <c r="BE19" s="19"/>
       <c r="BF19" s="13">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" ca="1" si="5"/>
         <v>46239</v>
       </c>
       <c r="BG19" s="12"/>
@@ -4821,7 +4752,7 @@
       <c r="BL19" s="21"/>
       <c r="BM19" s="19"/>
       <c r="BN19" s="13">
-        <f t="shared" ca="1" si="18"/>
+        <f t="shared" ca="1" si="6"/>
         <v>46270</v>
       </c>
       <c r="BO19" s="12"/>
@@ -4832,7 +4763,7 @@
       <c r="BT19" s="21"/>
       <c r="BU19" s="19"/>
       <c r="BV19" s="13">
-        <f t="shared" ca="1" si="19"/>
+        <f t="shared" ca="1" si="7"/>
         <v>46300</v>
       </c>
       <c r="BW19" s="12"/>
@@ -4843,7 +4774,7 @@
       <c r="CB19" s="21"/>
       <c r="CC19" s="19"/>
       <c r="CD19" s="13">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" ca="1" si="8"/>
         <v>46331</v>
       </c>
       <c r="CE19" s="12"/>
@@ -4854,7 +4785,7 @@
       <c r="CJ19" s="21"/>
       <c r="CK19" s="19"/>
       <c r="CL19" s="13">
-        <f t="shared" ca="1" si="21"/>
+        <f t="shared" ca="1" si="9"/>
         <v>46361</v>
       </c>
       <c r="CM19" s="12"/>
@@ -4868,7 +4799,7 @@
     <row r="20" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
       <c r="B20" s="13">
-        <f t="shared" ca="1" si="22"/>
+        <f t="shared" ca="1" si="10"/>
         <v>46028</v>
       </c>
       <c r="C20" s="12"/>
@@ -4879,7 +4810,7 @@
       <c r="H20" s="21"/>
       <c r="I20" s="19"/>
       <c r="J20" s="13">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" ca="1" si="11"/>
         <v>46059</v>
       </c>
       <c r="K20" s="12"/>
@@ -4890,7 +4821,7 @@
       <c r="P20" s="21"/>
       <c r="Q20" s="19"/>
       <c r="R20" s="13">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="0"/>
         <v>46087</v>
       </c>
       <c r="S20" s="12"/>
@@ -4901,7 +4832,7 @@
       <c r="X20" s="21"/>
       <c r="Y20" s="19"/>
       <c r="Z20" s="13">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" ca="1" si="1"/>
         <v>46118</v>
       </c>
       <c r="AA20" s="12"/>
@@ -4912,7 +4843,7 @@
       <c r="AF20" s="21"/>
       <c r="AG20" s="19"/>
       <c r="AH20" s="13">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" ca="1" si="2"/>
         <v>46148</v>
       </c>
       <c r="AI20" s="12"/>
@@ -4923,7 +4854,7 @@
       <c r="AN20" s="21"/>
       <c r="AO20" s="19"/>
       <c r="AP20" s="13">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="3"/>
         <v>46179</v>
       </c>
       <c r="AQ20" s="12"/>
@@ -4934,7 +4865,7 @@
       <c r="AV20" s="21"/>
       <c r="AW20" s="19"/>
       <c r="AX20" s="13">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="4"/>
         <v>46209</v>
       </c>
       <c r="AY20" s="12"/>
@@ -4945,7 +4876,7 @@
       <c r="BD20" s="21"/>
       <c r="BE20" s="19"/>
       <c r="BF20" s="13">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" ca="1" si="5"/>
         <v>46240</v>
       </c>
       <c r="BG20" s="12"/>
@@ -4956,7 +4887,7 @@
       <c r="BL20" s="21"/>
       <c r="BM20" s="19"/>
       <c r="BN20" s="13">
-        <f t="shared" ca="1" si="18"/>
+        <f t="shared" ca="1" si="6"/>
         <v>46271</v>
       </c>
       <c r="BO20" s="12"/>
@@ -4967,7 +4898,7 @@
       <c r="BT20" s="21"/>
       <c r="BU20" s="19"/>
       <c r="BV20" s="13">
-        <f t="shared" ca="1" si="19"/>
+        <f t="shared" ca="1" si="7"/>
         <v>46301</v>
       </c>
       <c r="BW20" s="12"/>
@@ -4978,7 +4909,7 @@
       <c r="CB20" s="21"/>
       <c r="CC20" s="19"/>
       <c r="CD20" s="13">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" ca="1" si="8"/>
         <v>46332</v>
       </c>
       <c r="CE20" s="12"/>
@@ -4989,7 +4920,7 @@
       <c r="CJ20" s="21"/>
       <c r="CK20" s="19"/>
       <c r="CL20" s="13">
-        <f t="shared" ca="1" si="21"/>
+        <f t="shared" ca="1" si="9"/>
         <v>46362</v>
       </c>
       <c r="CM20" s="12"/>
@@ -5003,7 +4934,7 @@
     <row r="21" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1"/>
       <c r="B21" s="13">
-        <f t="shared" ca="1" si="22"/>
+        <f t="shared" ca="1" si="10"/>
         <v>46029</v>
       </c>
       <c r="C21" s="12"/>
@@ -5014,7 +4945,7 @@
       <c r="H21" s="21"/>
       <c r="I21" s="19"/>
       <c r="J21" s="13">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" ca="1" si="11"/>
         <v>46060</v>
       </c>
       <c r="K21" s="12"/>
@@ -5025,7 +4956,7 @@
       <c r="P21" s="21"/>
       <c r="Q21" s="19"/>
       <c r="R21" s="13">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="0"/>
         <v>46088</v>
       </c>
       <c r="S21" s="12"/>
@@ -5036,7 +4967,7 @@
       <c r="X21" s="21"/>
       <c r="Y21" s="19"/>
       <c r="Z21" s="13">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" ca="1" si="1"/>
         <v>46119</v>
       </c>
       <c r="AA21" s="12"/>
@@ -5047,7 +4978,7 @@
       <c r="AF21" s="21"/>
       <c r="AG21" s="19"/>
       <c r="AH21" s="13">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" ca="1" si="2"/>
         <v>46149</v>
       </c>
       <c r="AI21" s="12"/>
@@ -5058,7 +4989,7 @@
       <c r="AN21" s="21"/>
       <c r="AO21" s="19"/>
       <c r="AP21" s="13">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="3"/>
         <v>46180</v>
       </c>
       <c r="AQ21" s="12"/>
@@ -5069,7 +5000,7 @@
       <c r="AV21" s="21"/>
       <c r="AW21" s="19"/>
       <c r="AX21" s="13">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="4"/>
         <v>46210</v>
       </c>
       <c r="AY21" s="12"/>
@@ -5080,7 +5011,7 @@
       <c r="BD21" s="21"/>
       <c r="BE21" s="19"/>
       <c r="BF21" s="13">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" ca="1" si="5"/>
         <v>46241</v>
       </c>
       <c r="BG21" s="12"/>
@@ -5091,7 +5022,7 @@
       <c r="BL21" s="21"/>
       <c r="BM21" s="19"/>
       <c r="BN21" s="13">
-        <f t="shared" ca="1" si="18"/>
+        <f t="shared" ca="1" si="6"/>
         <v>46272</v>
       </c>
       <c r="BO21" s="12"/>
@@ -5102,7 +5033,7 @@
       <c r="BT21" s="21"/>
       <c r="BU21" s="19"/>
       <c r="BV21" s="13">
-        <f t="shared" ca="1" si="19"/>
+        <f t="shared" ca="1" si="7"/>
         <v>46302</v>
       </c>
       <c r="BW21" s="12" t="s">
@@ -5115,7 +5046,7 @@
       <c r="CB21" s="21"/>
       <c r="CC21" s="19"/>
       <c r="CD21" s="13">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" ca="1" si="8"/>
         <v>46333</v>
       </c>
       <c r="CE21" s="12"/>
@@ -5126,7 +5057,7 @@
       <c r="CJ21" s="21"/>
       <c r="CK21" s="19"/>
       <c r="CL21" s="13">
-        <f t="shared" ca="1" si="21"/>
+        <f t="shared" ca="1" si="9"/>
         <v>46363</v>
       </c>
       <c r="CM21" s="12"/>
@@ -5140,7 +5071,7 @@
     <row r="22" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1"/>
       <c r="B22" s="13">
-        <f t="shared" ref="B22:B31" ca="1" si="24">B21+1</f>
+        <f t="shared" ref="B22:B31" ca="1" si="12">B21+1</f>
         <v>46030</v>
       </c>
       <c r="C22" s="12"/>
@@ -5151,7 +5082,7 @@
       <c r="H22" s="21"/>
       <c r="I22" s="19"/>
       <c r="J22" s="13">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" ca="1" si="11"/>
         <v>46061</v>
       </c>
       <c r="K22" s="12"/>
@@ -5162,7 +5093,7 @@
       <c r="P22" s="21"/>
       <c r="Q22" s="19"/>
       <c r="R22" s="13">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="0"/>
         <v>46089</v>
       </c>
       <c r="S22" s="12"/>
@@ -5173,7 +5104,7 @@
       <c r="X22" s="21"/>
       <c r="Y22" s="19"/>
       <c r="Z22" s="13">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" ca="1" si="1"/>
         <v>46120</v>
       </c>
       <c r="AA22" s="12"/>
@@ -5184,7 +5115,7 @@
       <c r="AF22" s="21"/>
       <c r="AG22" s="19"/>
       <c r="AH22" s="13">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" ca="1" si="2"/>
         <v>46150</v>
       </c>
       <c r="AI22" s="12" t="s">
@@ -5197,7 +5128,7 @@
       <c r="AN22" s="21"/>
       <c r="AO22" s="19"/>
       <c r="AP22" s="13">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="3"/>
         <v>46181</v>
       </c>
       <c r="AQ22" s="12"/>
@@ -5208,7 +5139,7 @@
       <c r="AV22" s="21"/>
       <c r="AW22" s="19"/>
       <c r="AX22" s="13">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="4"/>
         <v>46211</v>
       </c>
       <c r="AY22" s="12"/>
@@ -5219,7 +5150,7 @@
       <c r="BD22" s="21"/>
       <c r="BE22" s="19"/>
       <c r="BF22" s="13">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" ca="1" si="5"/>
         <v>46242</v>
       </c>
       <c r="BG22" s="12"/>
@@ -5230,7 +5161,7 @@
       <c r="BL22" s="21"/>
       <c r="BM22" s="19"/>
       <c r="BN22" s="13">
-        <f t="shared" ca="1" si="18"/>
+        <f t="shared" ca="1" si="6"/>
         <v>46273</v>
       </c>
       <c r="BO22" s="12"/>
@@ -5241,7 +5172,7 @@
       <c r="BT22" s="21"/>
       <c r="BU22" s="19"/>
       <c r="BV22" s="13">
-        <f t="shared" ca="1" si="19"/>
+        <f t="shared" ca="1" si="7"/>
         <v>46303</v>
       </c>
       <c r="BW22" s="12"/>
@@ -5252,7 +5183,7 @@
       <c r="CB22" s="21"/>
       <c r="CC22" s="19"/>
       <c r="CD22" s="13">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" ca="1" si="8"/>
         <v>46334</v>
       </c>
       <c r="CE22" s="12"/>
@@ -5263,7 +5194,7 @@
       <c r="CJ22" s="21"/>
       <c r="CK22" s="19"/>
       <c r="CL22" s="13">
-        <f t="shared" ca="1" si="21"/>
+        <f t="shared" ca="1" si="9"/>
         <v>46364</v>
       </c>
       <c r="CM22" s="12"/>
@@ -5277,7 +5208,7 @@
     <row r="23" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1"/>
       <c r="B23" s="13">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" ca="1" si="12"/>
         <v>46031</v>
       </c>
       <c r="C23" s="12"/>
@@ -5288,7 +5219,7 @@
       <c r="H23" s="21"/>
       <c r="I23" s="19"/>
       <c r="J23" s="13">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" ca="1" si="11"/>
         <v>46062</v>
       </c>
       <c r="K23" s="12"/>
@@ -5299,7 +5230,7 @@
       <c r="P23" s="21"/>
       <c r="Q23" s="19"/>
       <c r="R23" s="13">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="0"/>
         <v>46090</v>
       </c>
       <c r="S23" s="12"/>
@@ -5310,7 +5241,7 @@
       <c r="X23" s="21"/>
       <c r="Y23" s="19"/>
       <c r="Z23" s="13">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" ca="1" si="1"/>
         <v>46121</v>
       </c>
       <c r="AA23" s="12"/>
@@ -5321,7 +5252,7 @@
       <c r="AF23" s="21"/>
       <c r="AG23" s="19"/>
       <c r="AH23" s="13">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" ca="1" si="2"/>
         <v>46151</v>
       </c>
       <c r="AI23" s="12"/>
@@ -5332,7 +5263,7 @@
       <c r="AN23" s="21"/>
       <c r="AO23" s="19"/>
       <c r="AP23" s="13">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="3"/>
         <v>46182</v>
       </c>
       <c r="AQ23" s="12"/>
@@ -5343,7 +5274,7 @@
       <c r="AV23" s="21"/>
       <c r="AW23" s="19"/>
       <c r="AX23" s="13">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="4"/>
         <v>46212</v>
       </c>
       <c r="AY23" s="12"/>
@@ -5354,7 +5285,7 @@
       <c r="BD23" s="21"/>
       <c r="BE23" s="19"/>
       <c r="BF23" s="13">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" ca="1" si="5"/>
         <v>46243</v>
       </c>
       <c r="BG23" s="12"/>
@@ -5365,7 +5296,7 @@
       <c r="BL23" s="21"/>
       <c r="BM23" s="19"/>
       <c r="BN23" s="13">
-        <f t="shared" ca="1" si="18"/>
+        <f t="shared" ca="1" si="6"/>
         <v>46274</v>
       </c>
       <c r="BO23" s="12"/>
@@ -5376,7 +5307,7 @@
       <c r="BT23" s="21"/>
       <c r="BU23" s="19"/>
       <c r="BV23" s="13">
-        <f t="shared" ca="1" si="19"/>
+        <f t="shared" ca="1" si="7"/>
         <v>46304</v>
       </c>
       <c r="BW23" s="12"/>
@@ -5387,7 +5318,7 @@
       <c r="CB23" s="21"/>
       <c r="CC23" s="19"/>
       <c r="CD23" s="13">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" ca="1" si="8"/>
         <v>46335</v>
       </c>
       <c r="CE23" s="12"/>
@@ -5398,7 +5329,7 @@
       <c r="CJ23" s="21"/>
       <c r="CK23" s="19"/>
       <c r="CL23" s="13">
-        <f t="shared" ca="1" si="21"/>
+        <f t="shared" ca="1" si="9"/>
         <v>46365</v>
       </c>
       <c r="CM23" s="12"/>
@@ -5412,7 +5343,7 @@
     <row r="24" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1"/>
       <c r="B24" s="13">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" ca="1" si="12"/>
         <v>46032</v>
       </c>
       <c r="C24" s="12"/>
@@ -5423,7 +5354,7 @@
       <c r="H24" s="21"/>
       <c r="I24" s="19"/>
       <c r="J24" s="13">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" ca="1" si="11"/>
         <v>46063</v>
       </c>
       <c r="K24" s="12"/>
@@ -5434,7 +5365,7 @@
       <c r="P24" s="21"/>
       <c r="Q24" s="19"/>
       <c r="R24" s="13">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="0"/>
         <v>46091</v>
       </c>
       <c r="S24" s="12"/>
@@ -5445,7 +5376,7 @@
       <c r="X24" s="21"/>
       <c r="Y24" s="19"/>
       <c r="Z24" s="13">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" ca="1" si="1"/>
         <v>46122</v>
       </c>
       <c r="AA24" s="12"/>
@@ -5456,7 +5387,7 @@
       <c r="AF24" s="21"/>
       <c r="AG24" s="19"/>
       <c r="AH24" s="13">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" ca="1" si="2"/>
         <v>46152</v>
       </c>
       <c r="AI24" s="12"/>
@@ -5467,7 +5398,7 @@
       <c r="AN24" s="21"/>
       <c r="AO24" s="19"/>
       <c r="AP24" s="13">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="3"/>
         <v>46183</v>
       </c>
       <c r="AQ24" s="12"/>
@@ -5478,7 +5409,7 @@
       <c r="AV24" s="21"/>
       <c r="AW24" s="19"/>
       <c r="AX24" s="13">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="4"/>
         <v>46213</v>
       </c>
       <c r="AY24" s="12"/>
@@ -5489,7 +5420,7 @@
       <c r="BD24" s="21"/>
       <c r="BE24" s="19"/>
       <c r="BF24" s="13">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" ca="1" si="5"/>
         <v>46244</v>
       </c>
       <c r="BG24" s="12"/>
@@ -5500,7 +5431,7 @@
       <c r="BL24" s="21"/>
       <c r="BM24" s="19"/>
       <c r="BN24" s="13">
-        <f t="shared" ca="1" si="18"/>
+        <f t="shared" ca="1" si="6"/>
         <v>46275</v>
       </c>
       <c r="BO24" s="12"/>
@@ -5511,7 +5442,7 @@
       <c r="BT24" s="21"/>
       <c r="BU24" s="19"/>
       <c r="BV24" s="13">
-        <f t="shared" ca="1" si="19"/>
+        <f t="shared" ca="1" si="7"/>
         <v>46305</v>
       </c>
       <c r="BW24" s="12"/>
@@ -5522,7 +5453,7 @@
       <c r="CB24" s="21"/>
       <c r="CC24" s="19"/>
       <c r="CD24" s="13">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" ca="1" si="8"/>
         <v>46336</v>
       </c>
       <c r="CE24" s="12"/>
@@ -5533,7 +5464,7 @@
       <c r="CJ24" s="21"/>
       <c r="CK24" s="19"/>
       <c r="CL24" s="13">
-        <f t="shared" ca="1" si="21"/>
+        <f t="shared" ca="1" si="9"/>
         <v>46366</v>
       </c>
       <c r="CM24" s="12"/>
@@ -5547,7 +5478,7 @@
     <row r="25" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1"/>
       <c r="B25" s="13">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" ca="1" si="12"/>
         <v>46033</v>
       </c>
       <c r="C25" s="12"/>
@@ -5558,7 +5489,7 @@
       <c r="H25" s="21"/>
       <c r="I25" s="19"/>
       <c r="J25" s="13">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" ca="1" si="11"/>
         <v>46064</v>
       </c>
       <c r="K25" s="12"/>
@@ -5569,7 +5500,7 @@
       <c r="P25" s="21"/>
       <c r="Q25" s="19"/>
       <c r="R25" s="13">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="0"/>
         <v>46092</v>
       </c>
       <c r="S25" s="12"/>
@@ -5580,7 +5511,7 @@
       <c r="X25" s="21"/>
       <c r="Y25" s="19"/>
       <c r="Z25" s="13">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" ca="1" si="1"/>
         <v>46123</v>
       </c>
       <c r="AA25" s="12"/>
@@ -5591,7 +5522,7 @@
       <c r="AF25" s="21"/>
       <c r="AG25" s="19"/>
       <c r="AH25" s="13">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" ca="1" si="2"/>
         <v>46153</v>
       </c>
       <c r="AI25" s="12"/>
@@ -5602,7 +5533,7 @@
       <c r="AN25" s="21"/>
       <c r="AO25" s="19"/>
       <c r="AP25" s="13">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="3"/>
         <v>46184</v>
       </c>
       <c r="AQ25" s="12"/>
@@ -5613,7 +5544,7 @@
       <c r="AV25" s="21"/>
       <c r="AW25" s="19"/>
       <c r="AX25" s="13">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="4"/>
         <v>46214</v>
       </c>
       <c r="AY25" s="12"/>
@@ -5624,7 +5555,7 @@
       <c r="BD25" s="21"/>
       <c r="BE25" s="19"/>
       <c r="BF25" s="13">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" ca="1" si="5"/>
         <v>46245</v>
       </c>
       <c r="BG25" s="12"/>
@@ -5635,7 +5566,7 @@
       <c r="BL25" s="21"/>
       <c r="BM25" s="19"/>
       <c r="BN25" s="13">
-        <f t="shared" ca="1" si="18"/>
+        <f t="shared" ca="1" si="6"/>
         <v>46276</v>
       </c>
       <c r="BO25" s="12"/>
@@ -5646,7 +5577,7 @@
       <c r="BT25" s="21"/>
       <c r="BU25" s="19"/>
       <c r="BV25" s="13">
-        <f t="shared" ca="1" si="19"/>
+        <f t="shared" ca="1" si="7"/>
         <v>46306</v>
       </c>
       <c r="BW25" s="12"/>
@@ -5657,7 +5588,7 @@
       <c r="CB25" s="21"/>
       <c r="CC25" s="19"/>
       <c r="CD25" s="13">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" ca="1" si="8"/>
         <v>46337</v>
       </c>
       <c r="CE25" s="12"/>
@@ -5668,7 +5599,7 @@
       <c r="CJ25" s="21"/>
       <c r="CK25" s="19"/>
       <c r="CL25" s="13">
-        <f t="shared" ca="1" si="21"/>
+        <f t="shared" ca="1" si="9"/>
         <v>46367</v>
       </c>
       <c r="CM25" s="12"/>
@@ -5682,7 +5613,7 @@
     <row r="26" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1"/>
       <c r="B26" s="13">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" ca="1" si="12"/>
         <v>46034</v>
       </c>
       <c r="C26" s="12"/>
@@ -5693,7 +5624,7 @@
       <c r="H26" s="21"/>
       <c r="I26" s="19"/>
       <c r="J26" s="13">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" ca="1" si="11"/>
         <v>46065</v>
       </c>
       <c r="K26" s="12"/>
@@ -5704,7 +5635,7 @@
       <c r="P26" s="21"/>
       <c r="Q26" s="19"/>
       <c r="R26" s="13">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="0"/>
         <v>46093</v>
       </c>
       <c r="S26" s="12"/>
@@ -5715,7 +5646,7 @@
       <c r="X26" s="21"/>
       <c r="Y26" s="19"/>
       <c r="Z26" s="13">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" ca="1" si="1"/>
         <v>46124</v>
       </c>
       <c r="AA26" s="12"/>
@@ -5726,7 +5657,7 @@
       <c r="AF26" s="21"/>
       <c r="AG26" s="19"/>
       <c r="AH26" s="13">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" ca="1" si="2"/>
         <v>46154</v>
       </c>
       <c r="AI26" s="12"/>
@@ -5737,7 +5668,7 @@
       <c r="AN26" s="21"/>
       <c r="AO26" s="19"/>
       <c r="AP26" s="13">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="3"/>
         <v>46185</v>
       </c>
       <c r="AQ26" s="12"/>
@@ -5748,7 +5679,7 @@
       <c r="AV26" s="21"/>
       <c r="AW26" s="19"/>
       <c r="AX26" s="13">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="4"/>
         <v>46215</v>
       </c>
       <c r="AY26" s="12"/>
@@ -5759,7 +5690,7 @@
       <c r="BD26" s="21"/>
       <c r="BE26" s="19"/>
       <c r="BF26" s="13">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" ca="1" si="5"/>
         <v>46246</v>
       </c>
       <c r="BG26" s="12"/>
@@ -5770,7 +5701,7 @@
       <c r="BL26" s="21"/>
       <c r="BM26" s="19"/>
       <c r="BN26" s="13">
-        <f t="shared" ca="1" si="18"/>
+        <f t="shared" ca="1" si="6"/>
         <v>46277</v>
       </c>
       <c r="BO26" s="12"/>
@@ -5781,7 +5712,7 @@
       <c r="BT26" s="21"/>
       <c r="BU26" s="19"/>
       <c r="BV26" s="13">
-        <f t="shared" ca="1" si="19"/>
+        <f t="shared" ca="1" si="7"/>
         <v>46307</v>
       </c>
       <c r="BW26" s="12"/>
@@ -5792,7 +5723,7 @@
       <c r="CB26" s="21"/>
       <c r="CC26" s="19"/>
       <c r="CD26" s="13">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" ca="1" si="8"/>
         <v>46338</v>
       </c>
       <c r="CE26" s="12"/>
@@ -5803,7 +5734,7 @@
       <c r="CJ26" s="21"/>
       <c r="CK26" s="19"/>
       <c r="CL26" s="13">
-        <f t="shared" ca="1" si="21"/>
+        <f t="shared" ca="1" si="9"/>
         <v>46368</v>
       </c>
       <c r="CM26" s="12"/>
@@ -5817,7 +5748,7 @@
     <row r="27" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1"/>
       <c r="B27" s="13">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" ca="1" si="12"/>
         <v>46035</v>
       </c>
       <c r="C27" s="12"/>
@@ -5828,7 +5759,7 @@
       <c r="H27" s="21"/>
       <c r="I27" s="19"/>
       <c r="J27" s="13">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" ca="1" si="11"/>
         <v>46066</v>
       </c>
       <c r="K27" s="12"/>
@@ -5839,7 +5770,7 @@
       <c r="P27" s="21"/>
       <c r="Q27" s="19"/>
       <c r="R27" s="13">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="0"/>
         <v>46094</v>
       </c>
       <c r="S27" s="12"/>
@@ -5850,7 +5781,7 @@
       <c r="X27" s="21"/>
       <c r="Y27" s="19"/>
       <c r="Z27" s="13">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" ca="1" si="1"/>
         <v>46125</v>
       </c>
       <c r="AA27" s="12"/>
@@ -5861,7 +5792,7 @@
       <c r="AF27" s="21"/>
       <c r="AG27" s="19"/>
       <c r="AH27" s="13">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" ca="1" si="2"/>
         <v>46155</v>
       </c>
       <c r="AI27" s="12"/>
@@ -5872,7 +5803,7 @@
       <c r="AN27" s="21"/>
       <c r="AO27" s="19"/>
       <c r="AP27" s="13">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="3"/>
         <v>46186</v>
       </c>
       <c r="AQ27" s="12"/>
@@ -5883,7 +5814,7 @@
       <c r="AV27" s="21"/>
       <c r="AW27" s="19"/>
       <c r="AX27" s="13">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="4"/>
         <v>46216</v>
       </c>
       <c r="AY27" s="12"/>
@@ -5894,7 +5825,7 @@
       <c r="BD27" s="21"/>
       <c r="BE27" s="19"/>
       <c r="BF27" s="13">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" ca="1" si="5"/>
         <v>46247</v>
       </c>
       <c r="BG27" s="12"/>
@@ -5905,7 +5836,7 @@
       <c r="BL27" s="21"/>
       <c r="BM27" s="19"/>
       <c r="BN27" s="13">
-        <f t="shared" ca="1" si="18"/>
+        <f t="shared" ca="1" si="6"/>
         <v>46278</v>
       </c>
       <c r="BO27" s="12"/>
@@ -5916,7 +5847,7 @@
       <c r="BT27" s="21"/>
       <c r="BU27" s="19"/>
       <c r="BV27" s="13">
-        <f t="shared" ca="1" si="19"/>
+        <f t="shared" ca="1" si="7"/>
         <v>46308</v>
       </c>
       <c r="BW27" s="12"/>
@@ -5927,7 +5858,7 @@
       <c r="CB27" s="21"/>
       <c r="CC27" s="19"/>
       <c r="CD27" s="13">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" ca="1" si="8"/>
         <v>46339</v>
       </c>
       <c r="CE27" s="12"/>
@@ -5938,7 +5869,7 @@
       <c r="CJ27" s="21"/>
       <c r="CK27" s="19"/>
       <c r="CL27" s="13">
-        <f t="shared" ca="1" si="21"/>
+        <f t="shared" ca="1" si="9"/>
         <v>46369</v>
       </c>
       <c r="CM27" s="12"/>
@@ -5952,7 +5883,7 @@
     <row r="28" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1"/>
       <c r="B28" s="13">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" ca="1" si="12"/>
         <v>46036</v>
       </c>
       <c r="C28" s="12"/>
@@ -5963,7 +5894,7 @@
       <c r="H28" s="21"/>
       <c r="I28" s="19"/>
       <c r="J28" s="13">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" ca="1" si="11"/>
         <v>46067</v>
       </c>
       <c r="K28" s="12"/>
@@ -5974,7 +5905,7 @@
       <c r="P28" s="21"/>
       <c r="Q28" s="19"/>
       <c r="R28" s="13">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="0"/>
         <v>46095</v>
       </c>
       <c r="S28" s="12" t="s">
@@ -5987,7 +5918,7 @@
       <c r="X28" s="21"/>
       <c r="Y28" s="19"/>
       <c r="Z28" s="13">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" ca="1" si="1"/>
         <v>46126</v>
       </c>
       <c r="AA28" s="12"/>
@@ -5998,7 +5929,7 @@
       <c r="AF28" s="21"/>
       <c r="AG28" s="19"/>
       <c r="AH28" s="13">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" ca="1" si="2"/>
         <v>46156</v>
       </c>
       <c r="AI28" s="12"/>
@@ -6009,7 +5940,7 @@
       <c r="AN28" s="21"/>
       <c r="AO28" s="19"/>
       <c r="AP28" s="13">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="3"/>
         <v>46187</v>
       </c>
       <c r="AQ28" s="12"/>
@@ -6020,7 +5951,7 @@
       <c r="AV28" s="21"/>
       <c r="AW28" s="19"/>
       <c r="AX28" s="13">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="4"/>
         <v>46217</v>
       </c>
       <c r="AY28" s="12"/>
@@ -6031,7 +5962,7 @@
       <c r="BD28" s="21"/>
       <c r="BE28" s="19"/>
       <c r="BF28" s="13">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" ca="1" si="5"/>
         <v>46248</v>
       </c>
       <c r="BG28" s="12"/>
@@ -6042,7 +5973,7 @@
       <c r="BL28" s="21"/>
       <c r="BM28" s="19"/>
       <c r="BN28" s="13">
-        <f t="shared" ca="1" si="18"/>
+        <f t="shared" ca="1" si="6"/>
         <v>46279</v>
       </c>
       <c r="BO28" s="12"/>
@@ -6053,7 +5984,7 @@
       <c r="BT28" s="21"/>
       <c r="BU28" s="19"/>
       <c r="BV28" s="13">
-        <f t="shared" ca="1" si="19"/>
+        <f t="shared" ca="1" si="7"/>
         <v>46309</v>
       </c>
       <c r="BW28" s="12"/>
@@ -6064,7 +5995,7 @@
       <c r="CB28" s="21"/>
       <c r="CC28" s="19"/>
       <c r="CD28" s="13">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" ca="1" si="8"/>
         <v>46340</v>
       </c>
       <c r="CE28" s="12"/>
@@ -6075,7 +6006,7 @@
       <c r="CJ28" s="21"/>
       <c r="CK28" s="19"/>
       <c r="CL28" s="13">
-        <f t="shared" ca="1" si="21"/>
+        <f t="shared" ca="1" si="9"/>
         <v>46370</v>
       </c>
       <c r="CM28" s="12"/>
@@ -6089,7 +6020,7 @@
     <row r="29" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1"/>
       <c r="B29" s="13">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" ca="1" si="12"/>
         <v>46037</v>
       </c>
       <c r="C29" s="12"/>
@@ -6100,7 +6031,7 @@
       <c r="H29" s="21"/>
       <c r="I29" s="19"/>
       <c r="J29" s="13">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" ca="1" si="11"/>
         <v>46068</v>
       </c>
       <c r="K29" s="12"/>
@@ -6111,7 +6042,7 @@
       <c r="P29" s="21"/>
       <c r="Q29" s="19"/>
       <c r="R29" s="13">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="0"/>
         <v>46096</v>
       </c>
       <c r="S29" s="12"/>
@@ -6122,7 +6053,7 @@
       <c r="X29" s="21"/>
       <c r="Y29" s="19"/>
       <c r="Z29" s="13">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" ca="1" si="1"/>
         <v>46127</v>
       </c>
       <c r="AA29" s="12"/>
@@ -6133,7 +6064,7 @@
       <c r="AF29" s="21"/>
       <c r="AG29" s="19"/>
       <c r="AH29" s="13">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" ca="1" si="2"/>
         <v>46157</v>
       </c>
       <c r="AI29" s="12"/>
@@ -6144,7 +6075,7 @@
       <c r="AN29" s="21"/>
       <c r="AO29" s="19"/>
       <c r="AP29" s="13">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="3"/>
         <v>46188</v>
       </c>
       <c r="AQ29" s="12"/>
@@ -6155,7 +6086,7 @@
       <c r="AV29" s="21"/>
       <c r="AW29" s="19"/>
       <c r="AX29" s="13">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="4"/>
         <v>46218</v>
       </c>
       <c r="AY29" s="12"/>
@@ -6166,7 +6097,7 @@
       <c r="BD29" s="21"/>
       <c r="BE29" s="19"/>
       <c r="BF29" s="13">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" ca="1" si="5"/>
         <v>46249</v>
       </c>
       <c r="BG29" s="12"/>
@@ -6177,7 +6108,7 @@
       <c r="BL29" s="21"/>
       <c r="BM29" s="19"/>
       <c r="BN29" s="13">
-        <f t="shared" ca="1" si="18"/>
+        <f t="shared" ca="1" si="6"/>
         <v>46280</v>
       </c>
       <c r="BO29" s="12"/>
@@ -6188,7 +6119,7 @@
       <c r="BT29" s="21"/>
       <c r="BU29" s="19"/>
       <c r="BV29" s="13">
-        <f t="shared" ca="1" si="19"/>
+        <f t="shared" ca="1" si="7"/>
         <v>46310</v>
       </c>
       <c r="BW29" s="12"/>
@@ -6199,7 +6130,7 @@
       <c r="CB29" s="21"/>
       <c r="CC29" s="19"/>
       <c r="CD29" s="13">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" ca="1" si="8"/>
         <v>46341</v>
       </c>
       <c r="CE29" s="12"/>
@@ -6210,7 +6141,7 @@
       <c r="CJ29" s="21"/>
       <c r="CK29" s="19"/>
       <c r="CL29" s="13">
-        <f t="shared" ca="1" si="21"/>
+        <f t="shared" ca="1" si="9"/>
         <v>46371</v>
       </c>
       <c r="CM29" s="12"/>
@@ -6224,7 +6155,7 @@
     <row r="30" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1"/>
       <c r="B30" s="13">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" ca="1" si="12"/>
         <v>46038</v>
       </c>
       <c r="C30" s="12"/>
@@ -6235,7 +6166,7 @@
       <c r="H30" s="21"/>
       <c r="I30" s="19"/>
       <c r="J30" s="13">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" ca="1" si="11"/>
         <v>46069</v>
       </c>
       <c r="K30" s="12"/>
@@ -6246,7 +6177,7 @@
       <c r="P30" s="21"/>
       <c r="Q30" s="19"/>
       <c r="R30" s="13">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="0"/>
         <v>46097</v>
       </c>
       <c r="S30" s="12"/>
@@ -6257,7 +6188,7 @@
       <c r="X30" s="21"/>
       <c r="Y30" s="19"/>
       <c r="Z30" s="13">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" ca="1" si="1"/>
         <v>46128</v>
       </c>
       <c r="AA30" s="12"/>
@@ -6268,7 +6199,7 @@
       <c r="AF30" s="21"/>
       <c r="AG30" s="19"/>
       <c r="AH30" s="13">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" ca="1" si="2"/>
         <v>46158</v>
       </c>
       <c r="AI30" s="12"/>
@@ -6279,7 +6210,7 @@
       <c r="AN30" s="21"/>
       <c r="AO30" s="19"/>
       <c r="AP30" s="13">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="3"/>
         <v>46189</v>
       </c>
       <c r="AQ30" s="12"/>
@@ -6290,7 +6221,7 @@
       <c r="AV30" s="21"/>
       <c r="AW30" s="19"/>
       <c r="AX30" s="13">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="4"/>
         <v>46219</v>
       </c>
       <c r="AY30" s="12"/>
@@ -6301,7 +6232,7 @@
       <c r="BD30" s="21"/>
       <c r="BE30" s="19"/>
       <c r="BF30" s="13">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" ca="1" si="5"/>
         <v>46250</v>
       </c>
       <c r="BG30" s="12"/>
@@ -6312,7 +6243,7 @@
       <c r="BL30" s="21"/>
       <c r="BM30" s="19"/>
       <c r="BN30" s="13">
-        <f t="shared" ca="1" si="18"/>
+        <f t="shared" ca="1" si="6"/>
         <v>46281</v>
       </c>
       <c r="BO30" s="12"/>
@@ -6323,7 +6254,7 @@
       <c r="BT30" s="21"/>
       <c r="BU30" s="19"/>
       <c r="BV30" s="13">
-        <f t="shared" ca="1" si="19"/>
+        <f t="shared" ca="1" si="7"/>
         <v>46311</v>
       </c>
       <c r="BW30" s="12"/>
@@ -6334,7 +6265,7 @@
       <c r="CB30" s="21"/>
       <c r="CC30" s="19"/>
       <c r="CD30" s="13">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" ca="1" si="8"/>
         <v>46342</v>
       </c>
       <c r="CE30" s="12"/>
@@ -6345,7 +6276,7 @@
       <c r="CJ30" s="21"/>
       <c r="CK30" s="19"/>
       <c r="CL30" s="13">
-        <f t="shared" ca="1" si="21"/>
+        <f t="shared" ca="1" si="9"/>
         <v>46372</v>
       </c>
       <c r="CM30" s="12"/>
@@ -6359,7 +6290,7 @@
     <row r="31" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1"/>
       <c r="B31" s="13">
-        <f t="shared" ca="1" si="24"/>
+        <f t="shared" ca="1" si="12"/>
         <v>46039</v>
       </c>
       <c r="C31" s="12"/>
@@ -6370,7 +6301,7 @@
       <c r="H31" s="21"/>
       <c r="I31" s="19"/>
       <c r="J31" s="13">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" ca="1" si="11"/>
         <v>46070</v>
       </c>
       <c r="K31" s="12"/>
@@ -6381,7 +6312,7 @@
       <c r="P31" s="21"/>
       <c r="Q31" s="19"/>
       <c r="R31" s="13">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="0"/>
         <v>46098</v>
       </c>
       <c r="S31" s="12"/>
@@ -6392,7 +6323,7 @@
       <c r="X31" s="21"/>
       <c r="Y31" s="19"/>
       <c r="Z31" s="13">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" ca="1" si="1"/>
         <v>46129</v>
       </c>
       <c r="AA31" s="12"/>
@@ -6403,7 +6334,7 @@
       <c r="AF31" s="21"/>
       <c r="AG31" s="19"/>
       <c r="AH31" s="13">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" ca="1" si="2"/>
         <v>46159</v>
       </c>
       <c r="AI31" s="12"/>
@@ -6414,7 +6345,7 @@
       <c r="AN31" s="21"/>
       <c r="AO31" s="19"/>
       <c r="AP31" s="13">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="3"/>
         <v>46190</v>
       </c>
       <c r="AQ31" s="12"/>
@@ -6425,7 +6356,7 @@
       <c r="AV31" s="21"/>
       <c r="AW31" s="19"/>
       <c r="AX31" s="13">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="4"/>
         <v>46220</v>
       </c>
       <c r="AY31" s="12"/>
@@ -6436,7 +6367,7 @@
       <c r="BD31" s="21"/>
       <c r="BE31" s="19"/>
       <c r="BF31" s="13">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" ca="1" si="5"/>
         <v>46251</v>
       </c>
       <c r="BG31" s="12"/>
@@ -6447,7 +6378,7 @@
       <c r="BL31" s="21"/>
       <c r="BM31" s="19"/>
       <c r="BN31" s="13">
-        <f t="shared" ca="1" si="18"/>
+        <f t="shared" ca="1" si="6"/>
         <v>46282</v>
       </c>
       <c r="BO31" s="12"/>
@@ -6458,7 +6389,7 @@
       <c r="BT31" s="21"/>
       <c r="BU31" s="19"/>
       <c r="BV31" s="13">
-        <f t="shared" ca="1" si="19"/>
+        <f t="shared" ca="1" si="7"/>
         <v>46312</v>
       </c>
       <c r="BW31" s="12"/>
@@ -6469,7 +6400,7 @@
       <c r="CB31" s="21"/>
       <c r="CC31" s="19"/>
       <c r="CD31" s="13">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" ca="1" si="8"/>
         <v>46343</v>
       </c>
       <c r="CE31" s="12"/>
@@ -6480,7 +6411,7 @@
       <c r="CJ31" s="21"/>
       <c r="CK31" s="19"/>
       <c r="CL31" s="13">
-        <f t="shared" ca="1" si="21"/>
+        <f t="shared" ca="1" si="9"/>
         <v>46373</v>
       </c>
       <c r="CM31" s="12"/>
@@ -6494,7 +6425,7 @@
     <row r="32" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1"/>
       <c r="B32" s="13">
-        <f t="shared" ref="B32:B45" ca="1" si="25">B31+1</f>
+        <f t="shared" ref="B32:B45" ca="1" si="13">B31+1</f>
         <v>46040</v>
       </c>
       <c r="C32" s="12"/>
@@ -6505,7 +6436,7 @@
       <c r="H32" s="21"/>
       <c r="I32" s="19"/>
       <c r="J32" s="13">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" ca="1" si="11"/>
         <v>46071</v>
       </c>
       <c r="K32" s="12"/>
@@ -6516,7 +6447,7 @@
       <c r="P32" s="21"/>
       <c r="Q32" s="19"/>
       <c r="R32" s="13">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="0"/>
         <v>46099</v>
       </c>
       <c r="S32" s="12"/>
@@ -6527,7 +6458,7 @@
       <c r="X32" s="21"/>
       <c r="Y32" s="19"/>
       <c r="Z32" s="13">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" ca="1" si="1"/>
         <v>46130</v>
       </c>
       <c r="AA32" s="12"/>
@@ -6538,7 +6469,7 @@
       <c r="AF32" s="21"/>
       <c r="AG32" s="19"/>
       <c r="AH32" s="13">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" ca="1" si="2"/>
         <v>46160</v>
       </c>
       <c r="AI32" s="12"/>
@@ -6549,7 +6480,7 @@
       <c r="AN32" s="21"/>
       <c r="AO32" s="19"/>
       <c r="AP32" s="13">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="3"/>
         <v>46191</v>
       </c>
       <c r="AQ32" s="12"/>
@@ -6560,7 +6491,7 @@
       <c r="AV32" s="21"/>
       <c r="AW32" s="19"/>
       <c r="AX32" s="13">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="4"/>
         <v>46221</v>
       </c>
       <c r="AY32" s="12"/>
@@ -6571,7 +6502,7 @@
       <c r="BD32" s="21"/>
       <c r="BE32" s="19"/>
       <c r="BF32" s="13">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" ca="1" si="5"/>
         <v>46252</v>
       </c>
       <c r="BG32" s="12"/>
@@ -6582,7 +6513,7 @@
       <c r="BL32" s="21"/>
       <c r="BM32" s="19"/>
       <c r="BN32" s="13">
-        <f t="shared" ca="1" si="18"/>
+        <f t="shared" ca="1" si="6"/>
         <v>46283</v>
       </c>
       <c r="BO32" s="12"/>
@@ -6593,7 +6524,7 @@
       <c r="BT32" s="21"/>
       <c r="BU32" s="19"/>
       <c r="BV32" s="13">
-        <f t="shared" ca="1" si="19"/>
+        <f t="shared" ca="1" si="7"/>
         <v>46313</v>
       </c>
       <c r="BW32" s="12"/>
@@ -6604,7 +6535,7 @@
       <c r="CB32" s="21"/>
       <c r="CC32" s="19"/>
       <c r="CD32" s="13">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" ca="1" si="8"/>
         <v>46344</v>
       </c>
       <c r="CE32" s="12"/>
@@ -6615,7 +6546,7 @@
       <c r="CJ32" s="21"/>
       <c r="CK32" s="19"/>
       <c r="CL32" s="13">
-        <f t="shared" ca="1" si="21"/>
+        <f t="shared" ca="1" si="9"/>
         <v>46374</v>
       </c>
       <c r="CM32" s="12"/>
@@ -6629,7 +6560,7 @@
     <row r="33" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1"/>
       <c r="B33" s="13">
-        <f t="shared" ca="1" si="25"/>
+        <f t="shared" ca="1" si="13"/>
         <v>46041</v>
       </c>
       <c r="C33" s="12"/>
@@ -6640,7 +6571,7 @@
       <c r="H33" s="21"/>
       <c r="I33" s="19"/>
       <c r="J33" s="13">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" ca="1" si="11"/>
         <v>46072</v>
       </c>
       <c r="K33" s="12"/>
@@ -6651,7 +6582,7 @@
       <c r="P33" s="21"/>
       <c r="Q33" s="19"/>
       <c r="R33" s="13">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="0"/>
         <v>46100</v>
       </c>
       <c r="S33" s="12"/>
@@ -6662,7 +6593,7 @@
       <c r="X33" s="21"/>
       <c r="Y33" s="19"/>
       <c r="Z33" s="13">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" ca="1" si="1"/>
         <v>46131</v>
       </c>
       <c r="AA33" s="12"/>
@@ -6673,7 +6604,7 @@
       <c r="AF33" s="21"/>
       <c r="AG33" s="19"/>
       <c r="AH33" s="13">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" ca="1" si="2"/>
         <v>46161</v>
       </c>
       <c r="AI33" s="12"/>
@@ -6684,7 +6615,7 @@
       <c r="AN33" s="21"/>
       <c r="AO33" s="19"/>
       <c r="AP33" s="13">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="3"/>
         <v>46192</v>
       </c>
       <c r="AQ33" s="12"/>
@@ -6695,7 +6626,7 @@
       <c r="AV33" s="21"/>
       <c r="AW33" s="19"/>
       <c r="AX33" s="13">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="4"/>
         <v>46222</v>
       </c>
       <c r="AY33" s="12"/>
@@ -6706,7 +6637,7 @@
       <c r="BD33" s="21"/>
       <c r="BE33" s="19"/>
       <c r="BF33" s="13">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" ca="1" si="5"/>
         <v>46253</v>
       </c>
       <c r="BG33" s="12"/>
@@ -6717,7 +6648,7 @@
       <c r="BL33" s="21"/>
       <c r="BM33" s="19"/>
       <c r="BN33" s="13">
-        <f t="shared" ca="1" si="18"/>
+        <f t="shared" ca="1" si="6"/>
         <v>46284</v>
       </c>
       <c r="BO33" s="12"/>
@@ -6728,7 +6659,7 @@
       <c r="BT33" s="21"/>
       <c r="BU33" s="19"/>
       <c r="BV33" s="13">
-        <f t="shared" ca="1" si="19"/>
+        <f t="shared" ca="1" si="7"/>
         <v>46314</v>
       </c>
       <c r="BW33" s="12"/>
@@ -6739,7 +6670,7 @@
       <c r="CB33" s="21"/>
       <c r="CC33" s="19"/>
       <c r="CD33" s="13">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" ca="1" si="8"/>
         <v>46345</v>
       </c>
       <c r="CE33" s="12"/>
@@ -6750,7 +6681,7 @@
       <c r="CJ33" s="21"/>
       <c r="CK33" s="19"/>
       <c r="CL33" s="13">
-        <f t="shared" ca="1" si="21"/>
+        <f t="shared" ca="1" si="9"/>
         <v>46375</v>
       </c>
       <c r="CM33" s="12"/>
@@ -6764,7 +6695,7 @@
     <row r="34" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="1"/>
       <c r="B34" s="13">
-        <f t="shared" ca="1" si="25"/>
+        <f t="shared" ca="1" si="13"/>
         <v>46042</v>
       </c>
       <c r="C34" s="12"/>
@@ -6775,7 +6706,7 @@
       <c r="H34" s="21"/>
       <c r="I34" s="19"/>
       <c r="J34" s="13">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" ca="1" si="11"/>
         <v>46073</v>
       </c>
       <c r="K34" s="12"/>
@@ -6786,7 +6717,7 @@
       <c r="P34" s="21"/>
       <c r="Q34" s="19"/>
       <c r="R34" s="13">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="0"/>
         <v>46101</v>
       </c>
       <c r="S34" s="12"/>
@@ -6797,7 +6728,7 @@
       <c r="X34" s="21"/>
       <c r="Y34" s="19"/>
       <c r="Z34" s="13">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" ca="1" si="1"/>
         <v>46132</v>
       </c>
       <c r="AA34" s="12"/>
@@ -6808,7 +6739,7 @@
       <c r="AF34" s="21"/>
       <c r="AG34" s="19"/>
       <c r="AH34" s="13">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" ca="1" si="2"/>
         <v>46162</v>
       </c>
       <c r="AI34" s="12"/>
@@ -6819,7 +6750,7 @@
       <c r="AN34" s="21"/>
       <c r="AO34" s="19"/>
       <c r="AP34" s="13">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="3"/>
         <v>46193</v>
       </c>
       <c r="AQ34" s="12"/>
@@ -6830,7 +6761,7 @@
       <c r="AV34" s="21"/>
       <c r="AW34" s="19"/>
       <c r="AX34" s="13">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="4"/>
         <v>46223</v>
       </c>
       <c r="AY34" s="12"/>
@@ -6841,7 +6772,7 @@
       <c r="BD34" s="21"/>
       <c r="BE34" s="19"/>
       <c r="BF34" s="13">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" ca="1" si="5"/>
         <v>46254</v>
       </c>
       <c r="BG34" s="12"/>
@@ -6852,7 +6783,7 @@
       <c r="BL34" s="21"/>
       <c r="BM34" s="19"/>
       <c r="BN34" s="13">
-        <f t="shared" ca="1" si="18"/>
+        <f t="shared" ca="1" si="6"/>
         <v>46285</v>
       </c>
       <c r="BO34" s="12"/>
@@ -6863,7 +6794,7 @@
       <c r="BT34" s="21"/>
       <c r="BU34" s="19"/>
       <c r="BV34" s="13">
-        <f t="shared" ca="1" si="19"/>
+        <f t="shared" ca="1" si="7"/>
         <v>46315</v>
       </c>
       <c r="BW34" s="12"/>
@@ -6874,7 +6805,7 @@
       <c r="CB34" s="21"/>
       <c r="CC34" s="19"/>
       <c r="CD34" s="13">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" ca="1" si="8"/>
         <v>46346</v>
       </c>
       <c r="CE34" s="12"/>
@@ -6885,7 +6816,7 @@
       <c r="CJ34" s="21"/>
       <c r="CK34" s="19"/>
       <c r="CL34" s="13">
-        <f t="shared" ca="1" si="21"/>
+        <f t="shared" ca="1" si="9"/>
         <v>46376</v>
       </c>
       <c r="CM34" s="12"/>
@@ -6899,7 +6830,7 @@
     <row r="35" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1"/>
       <c r="B35" s="13">
-        <f t="shared" ca="1" si="25"/>
+        <f t="shared" ca="1" si="13"/>
         <v>46043</v>
       </c>
       <c r="C35" s="12"/>
@@ -6910,7 +6841,7 @@
       <c r="H35" s="21"/>
       <c r="I35" s="19"/>
       <c r="J35" s="13">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" ca="1" si="11"/>
         <v>46074</v>
       </c>
       <c r="K35" s="12"/>
@@ -6921,7 +6852,7 @@
       <c r="P35" s="21"/>
       <c r="Q35" s="19"/>
       <c r="R35" s="13">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="0"/>
         <v>46102</v>
       </c>
       <c r="S35" s="12"/>
@@ -6932,7 +6863,7 @@
       <c r="X35" s="21"/>
       <c r="Y35" s="19"/>
       <c r="Z35" s="13">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" ca="1" si="1"/>
         <v>46133</v>
       </c>
       <c r="AA35" s="12"/>
@@ -6943,7 +6874,7 @@
       <c r="AF35" s="21"/>
       <c r="AG35" s="19"/>
       <c r="AH35" s="13">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" ca="1" si="2"/>
         <v>46163</v>
       </c>
       <c r="AI35" s="12"/>
@@ -6954,7 +6885,7 @@
       <c r="AN35" s="21"/>
       <c r="AO35" s="19"/>
       <c r="AP35" s="13">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="3"/>
         <v>46194</v>
       </c>
       <c r="AQ35" s="12"/>
@@ -6965,7 +6896,7 @@
       <c r="AV35" s="21"/>
       <c r="AW35" s="19"/>
       <c r="AX35" s="13">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="4"/>
         <v>46224</v>
       </c>
       <c r="AY35" s="12"/>
@@ -6976,7 +6907,7 @@
       <c r="BD35" s="21"/>
       <c r="BE35" s="19"/>
       <c r="BF35" s="13">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" ca="1" si="5"/>
         <v>46255</v>
       </c>
       <c r="BG35" s="12"/>
@@ -6987,7 +6918,7 @@
       <c r="BL35" s="21"/>
       <c r="BM35" s="19"/>
       <c r="BN35" s="13">
-        <f t="shared" ca="1" si="18"/>
+        <f t="shared" ca="1" si="6"/>
         <v>46286</v>
       </c>
       <c r="BO35" s="12"/>
@@ -6998,7 +6929,7 @@
       <c r="BT35" s="21"/>
       <c r="BU35" s="19"/>
       <c r="BV35" s="13">
-        <f t="shared" ca="1" si="19"/>
+        <f t="shared" ca="1" si="7"/>
         <v>46316</v>
       </c>
       <c r="BW35" s="12"/>
@@ -7009,7 +6940,7 @@
       <c r="CB35" s="21"/>
       <c r="CC35" s="19"/>
       <c r="CD35" s="13">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" ca="1" si="8"/>
         <v>46347</v>
       </c>
       <c r="CE35" s="12"/>
@@ -7020,7 +6951,7 @@
       <c r="CJ35" s="21"/>
       <c r="CK35" s="19"/>
       <c r="CL35" s="13">
-        <f t="shared" ca="1" si="21"/>
+        <f t="shared" ca="1" si="9"/>
         <v>46377</v>
       </c>
       <c r="CM35" s="12"/>
@@ -7034,7 +6965,7 @@
     <row r="36" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1"/>
       <c r="B36" s="13">
-        <f t="shared" ca="1" si="25"/>
+        <f t="shared" ca="1" si="13"/>
         <v>46044</v>
       </c>
       <c r="C36" s="12"/>
@@ -7045,7 +6976,7 @@
       <c r="H36" s="21"/>
       <c r="I36" s="19"/>
       <c r="J36" s="13">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" ca="1" si="11"/>
         <v>46075</v>
       </c>
       <c r="K36" s="12"/>
@@ -7056,7 +6987,7 @@
       <c r="P36" s="21"/>
       <c r="Q36" s="19"/>
       <c r="R36" s="13">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="0"/>
         <v>46103</v>
       </c>
       <c r="S36" s="12"/>
@@ -7067,7 +6998,7 @@
       <c r="X36" s="21"/>
       <c r="Y36" s="19"/>
       <c r="Z36" s="13">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" ca="1" si="1"/>
         <v>46134</v>
       </c>
       <c r="AA36" s="12"/>
@@ -7078,7 +7009,7 @@
       <c r="AF36" s="21"/>
       <c r="AG36" s="19"/>
       <c r="AH36" s="13">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" ca="1" si="2"/>
         <v>46164</v>
       </c>
       <c r="AI36" s="12"/>
@@ -7089,7 +7020,7 @@
       <c r="AN36" s="21"/>
       <c r="AO36" s="19"/>
       <c r="AP36" s="13">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="3"/>
         <v>46195</v>
       </c>
       <c r="AQ36" s="12"/>
@@ -7100,7 +7031,7 @@
       <c r="AV36" s="21"/>
       <c r="AW36" s="19"/>
       <c r="AX36" s="13">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="4"/>
         <v>46225</v>
       </c>
       <c r="AY36" s="12"/>
@@ -7111,7 +7042,7 @@
       <c r="BD36" s="21"/>
       <c r="BE36" s="19"/>
       <c r="BF36" s="13">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" ca="1" si="5"/>
         <v>46256</v>
       </c>
       <c r="BG36" s="12"/>
@@ -7122,7 +7053,7 @@
       <c r="BL36" s="21"/>
       <c r="BM36" s="19"/>
       <c r="BN36" s="13">
-        <f t="shared" ca="1" si="18"/>
+        <f t="shared" ca="1" si="6"/>
         <v>46287</v>
       </c>
       <c r="BO36" s="12"/>
@@ -7133,7 +7064,7 @@
       <c r="BT36" s="21"/>
       <c r="BU36" s="19"/>
       <c r="BV36" s="13">
-        <f t="shared" ca="1" si="19"/>
+        <f t="shared" ca="1" si="7"/>
         <v>46317</v>
       </c>
       <c r="BW36" s="12"/>
@@ -7144,7 +7075,7 @@
       <c r="CB36" s="21"/>
       <c r="CC36" s="19"/>
       <c r="CD36" s="13">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" ca="1" si="8"/>
         <v>46348</v>
       </c>
       <c r="CE36" s="12"/>
@@ -7155,7 +7086,7 @@
       <c r="CJ36" s="21"/>
       <c r="CK36" s="19"/>
       <c r="CL36" s="13">
-        <f t="shared" ca="1" si="21"/>
+        <f t="shared" ca="1" si="9"/>
         <v>46378</v>
       </c>
       <c r="CM36" s="12"/>
@@ -7169,7 +7100,7 @@
     <row r="37" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="1"/>
       <c r="B37" s="13">
-        <f t="shared" ca="1" si="25"/>
+        <f t="shared" ca="1" si="13"/>
         <v>46045</v>
       </c>
       <c r="C37" s="12"/>
@@ -7180,7 +7111,7 @@
       <c r="H37" s="21"/>
       <c r="I37" s="19"/>
       <c r="J37" s="13">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" ca="1" si="11"/>
         <v>46076</v>
       </c>
       <c r="K37" s="12"/>
@@ -7191,7 +7122,7 @@
       <c r="P37" s="21"/>
       <c r="Q37" s="19"/>
       <c r="R37" s="13">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="0"/>
         <v>46104</v>
       </c>
       <c r="S37" s="12"/>
@@ -7202,7 +7133,7 @@
       <c r="X37" s="21"/>
       <c r="Y37" s="19"/>
       <c r="Z37" s="13">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" ca="1" si="1"/>
         <v>46135</v>
       </c>
       <c r="AA37" s="12"/>
@@ -7213,7 +7144,7 @@
       <c r="AF37" s="21"/>
       <c r="AG37" s="19"/>
       <c r="AH37" s="13">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" ca="1" si="2"/>
         <v>46165</v>
       </c>
       <c r="AI37" s="12"/>
@@ -7224,7 +7155,7 @@
       <c r="AN37" s="21"/>
       <c r="AO37" s="19"/>
       <c r="AP37" s="13">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="3"/>
         <v>46196</v>
       </c>
       <c r="AQ37" s="12"/>
@@ -7235,7 +7166,7 @@
       <c r="AV37" s="21"/>
       <c r="AW37" s="19"/>
       <c r="AX37" s="13">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="4"/>
         <v>46226</v>
       </c>
       <c r="AY37" s="12"/>
@@ -7246,7 +7177,7 @@
       <c r="BD37" s="21"/>
       <c r="BE37" s="19"/>
       <c r="BF37" s="13">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" ca="1" si="5"/>
         <v>46257</v>
       </c>
       <c r="BG37" s="12"/>
@@ -7257,7 +7188,7 @@
       <c r="BL37" s="21"/>
       <c r="BM37" s="19"/>
       <c r="BN37" s="13">
-        <f t="shared" ca="1" si="18"/>
+        <f t="shared" ca="1" si="6"/>
         <v>46288</v>
       </c>
       <c r="BO37" s="12"/>
@@ -7268,7 +7199,7 @@
       <c r="BT37" s="21"/>
       <c r="BU37" s="19"/>
       <c r="BV37" s="13">
-        <f t="shared" ca="1" si="19"/>
+        <f t="shared" ca="1" si="7"/>
         <v>46318</v>
       </c>
       <c r="BW37" s="12"/>
@@ -7279,7 +7210,7 @@
       <c r="CB37" s="21"/>
       <c r="CC37" s="19"/>
       <c r="CD37" s="13">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" ca="1" si="8"/>
         <v>46349</v>
       </c>
       <c r="CE37" s="12"/>
@@ -7290,7 +7221,7 @@
       <c r="CJ37" s="21"/>
       <c r="CK37" s="19"/>
       <c r="CL37" s="13">
-        <f t="shared" ca="1" si="21"/>
+        <f t="shared" ca="1" si="9"/>
         <v>46379</v>
       </c>
       <c r="CM37" s="12"/>
@@ -7304,7 +7235,7 @@
     <row r="38" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="1"/>
       <c r="B38" s="13">
-        <f t="shared" ca="1" si="25"/>
+        <f t="shared" ca="1" si="13"/>
         <v>46046</v>
       </c>
       <c r="C38" s="12"/>
@@ -7315,7 +7246,7 @@
       <c r="H38" s="21"/>
       <c r="I38" s="19"/>
       <c r="J38" s="13">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" ca="1" si="11"/>
         <v>46077</v>
       </c>
       <c r="K38" s="12"/>
@@ -7326,7 +7257,7 @@
       <c r="P38" s="21"/>
       <c r="Q38" s="19"/>
       <c r="R38" s="13">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="0"/>
         <v>46105</v>
       </c>
       <c r="S38" s="12"/>
@@ -7337,7 +7268,7 @@
       <c r="X38" s="21"/>
       <c r="Y38" s="19"/>
       <c r="Z38" s="13">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" ca="1" si="1"/>
         <v>46136</v>
       </c>
       <c r="AA38" s="12"/>
@@ -7348,7 +7279,7 @@
       <c r="AF38" s="21"/>
       <c r="AG38" s="19"/>
       <c r="AH38" s="13">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" ca="1" si="2"/>
         <v>46166</v>
       </c>
       <c r="AI38" s="12"/>
@@ -7359,7 +7290,7 @@
       <c r="AN38" s="21"/>
       <c r="AO38" s="19"/>
       <c r="AP38" s="13">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="3"/>
         <v>46197</v>
       </c>
       <c r="AQ38" s="12"/>
@@ -7370,7 +7301,7 @@
       <c r="AV38" s="21"/>
       <c r="AW38" s="19"/>
       <c r="AX38" s="13">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="4"/>
         <v>46227</v>
       </c>
       <c r="AY38" s="12"/>
@@ -7381,7 +7312,7 @@
       <c r="BD38" s="21"/>
       <c r="BE38" s="19"/>
       <c r="BF38" s="13">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" ca="1" si="5"/>
         <v>46258</v>
       </c>
       <c r="BG38" s="12"/>
@@ -7392,7 +7323,7 @@
       <c r="BL38" s="21"/>
       <c r="BM38" s="19"/>
       <c r="BN38" s="13">
-        <f t="shared" ca="1" si="18"/>
+        <f t="shared" ca="1" si="6"/>
         <v>46289</v>
       </c>
       <c r="BO38" s="12"/>
@@ -7403,7 +7334,7 @@
       <c r="BT38" s="21"/>
       <c r="BU38" s="19"/>
       <c r="BV38" s="13">
-        <f t="shared" ca="1" si="19"/>
+        <f t="shared" ca="1" si="7"/>
         <v>46319</v>
       </c>
       <c r="BW38" s="12"/>
@@ -7414,7 +7345,7 @@
       <c r="CB38" s="21"/>
       <c r="CC38" s="19"/>
       <c r="CD38" s="13">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" ca="1" si="8"/>
         <v>46350</v>
       </c>
       <c r="CE38" s="12"/>
@@ -7425,7 +7356,7 @@
       <c r="CJ38" s="21"/>
       <c r="CK38" s="19"/>
       <c r="CL38" s="13">
-        <f t="shared" ca="1" si="21"/>
+        <f t="shared" ca="1" si="9"/>
         <v>46380</v>
       </c>
       <c r="CM38" s="12"/>
@@ -7439,7 +7370,7 @@
     <row r="39" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="1"/>
       <c r="B39" s="13">
-        <f t="shared" ca="1" si="25"/>
+        <f t="shared" ca="1" si="13"/>
         <v>46047</v>
       </c>
       <c r="C39" s="12"/>
@@ -7450,7 +7381,7 @@
       <c r="H39" s="21"/>
       <c r="I39" s="19"/>
       <c r="J39" s="13">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" ca="1" si="11"/>
         <v>46078</v>
       </c>
       <c r="K39" s="12"/>
@@ -7461,7 +7392,7 @@
       <c r="P39" s="21"/>
       <c r="Q39" s="19"/>
       <c r="R39" s="13">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="0"/>
         <v>46106</v>
       </c>
       <c r="S39" s="12"/>
@@ -7472,7 +7403,7 @@
       <c r="X39" s="21"/>
       <c r="Y39" s="19"/>
       <c r="Z39" s="13">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" ca="1" si="1"/>
         <v>46137</v>
       </c>
       <c r="AA39" s="12"/>
@@ -7483,7 +7414,7 @@
       <c r="AF39" s="21"/>
       <c r="AG39" s="19"/>
       <c r="AH39" s="13">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" ca="1" si="2"/>
         <v>46167</v>
       </c>
       <c r="AI39" s="12"/>
@@ -7494,7 +7425,7 @@
       <c r="AN39" s="21"/>
       <c r="AO39" s="19"/>
       <c r="AP39" s="13">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="3"/>
         <v>46198</v>
       </c>
       <c r="AQ39" s="12"/>
@@ -7505,7 +7436,7 @@
       <c r="AV39" s="21"/>
       <c r="AW39" s="19"/>
       <c r="AX39" s="13">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="4"/>
         <v>46228</v>
       </c>
       <c r="AY39" s="12"/>
@@ -7516,7 +7447,7 @@
       <c r="BD39" s="21"/>
       <c r="BE39" s="19"/>
       <c r="BF39" s="13">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" ca="1" si="5"/>
         <v>46259</v>
       </c>
       <c r="BG39" s="12"/>
@@ -7527,7 +7458,7 @@
       <c r="BL39" s="21"/>
       <c r="BM39" s="19"/>
       <c r="BN39" s="13">
-        <f t="shared" ca="1" si="18"/>
+        <f t="shared" ca="1" si="6"/>
         <v>46290</v>
       </c>
       <c r="BO39" s="12"/>
@@ -7538,7 +7469,7 @@
       <c r="BT39" s="21"/>
       <c r="BU39" s="19"/>
       <c r="BV39" s="13">
-        <f t="shared" ca="1" si="19"/>
+        <f t="shared" ca="1" si="7"/>
         <v>46320</v>
       </c>
       <c r="BW39" s="12"/>
@@ -7549,7 +7480,7 @@
       <c r="CB39" s="21"/>
       <c r="CC39" s="19"/>
       <c r="CD39" s="13">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" ca="1" si="8"/>
         <v>46351</v>
       </c>
       <c r="CE39" s="12"/>
@@ -7560,7 +7491,7 @@
       <c r="CJ39" s="21"/>
       <c r="CK39" s="19"/>
       <c r="CL39" s="13">
-        <f t="shared" ca="1" si="21"/>
+        <f t="shared" ca="1" si="9"/>
         <v>46381</v>
       </c>
       <c r="CM39" s="12"/>
@@ -7574,7 +7505,7 @@
     <row r="40" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="1"/>
       <c r="B40" s="13">
-        <f t="shared" ca="1" si="25"/>
+        <f t="shared" ca="1" si="13"/>
         <v>46048</v>
       </c>
       <c r="C40" s="12"/>
@@ -7585,7 +7516,7 @@
       <c r="H40" s="21"/>
       <c r="I40" s="19"/>
       <c r="J40" s="13">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" ca="1" si="11"/>
         <v>46079</v>
       </c>
       <c r="K40" s="12"/>
@@ -7596,7 +7527,7 @@
       <c r="P40" s="21"/>
       <c r="Q40" s="19"/>
       <c r="R40" s="13">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="0"/>
         <v>46107</v>
       </c>
       <c r="S40" s="12"/>
@@ -7607,7 +7538,7 @@
       <c r="X40" s="21"/>
       <c r="Y40" s="19"/>
       <c r="Z40" s="13">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" ca="1" si="1"/>
         <v>46138</v>
       </c>
       <c r="AA40" s="12"/>
@@ -7618,7 +7549,7 @@
       <c r="AF40" s="21"/>
       <c r="AG40" s="19"/>
       <c r="AH40" s="13">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" ca="1" si="2"/>
         <v>46168</v>
       </c>
       <c r="AI40" s="12"/>
@@ -7629,7 +7560,7 @@
       <c r="AN40" s="21"/>
       <c r="AO40" s="19"/>
       <c r="AP40" s="13">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="3"/>
         <v>46199</v>
       </c>
       <c r="AQ40" s="12"/>
@@ -7640,7 +7571,7 @@
       <c r="AV40" s="21"/>
       <c r="AW40" s="19"/>
       <c r="AX40" s="13">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="4"/>
         <v>46229</v>
       </c>
       <c r="AY40" s="12"/>
@@ -7651,7 +7582,7 @@
       <c r="BD40" s="21"/>
       <c r="BE40" s="19"/>
       <c r="BF40" s="13">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" ca="1" si="5"/>
         <v>46260</v>
       </c>
       <c r="BG40" s="12"/>
@@ -7662,7 +7593,7 @@
       <c r="BL40" s="21"/>
       <c r="BM40" s="19"/>
       <c r="BN40" s="13">
-        <f t="shared" ca="1" si="18"/>
+        <f t="shared" ca="1" si="6"/>
         <v>46291</v>
       </c>
       <c r="BO40" s="12"/>
@@ -7673,7 +7604,7 @@
       <c r="BT40" s="21"/>
       <c r="BU40" s="19"/>
       <c r="BV40" s="13">
-        <f t="shared" ca="1" si="19"/>
+        <f t="shared" ca="1" si="7"/>
         <v>46321</v>
       </c>
       <c r="BW40" s="12"/>
@@ -7684,7 +7615,7 @@
       <c r="CB40" s="21"/>
       <c r="CC40" s="19"/>
       <c r="CD40" s="13">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" ca="1" si="8"/>
         <v>46352</v>
       </c>
       <c r="CE40" s="12"/>
@@ -7695,7 +7626,7 @@
       <c r="CJ40" s="21"/>
       <c r="CK40" s="19"/>
       <c r="CL40" s="13">
-        <f t="shared" ca="1" si="21"/>
+        <f t="shared" ca="1" si="9"/>
         <v>46382</v>
       </c>
       <c r="CM40" s="12"/>
@@ -7709,7 +7640,7 @@
     <row r="41" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="1"/>
       <c r="B41" s="13">
-        <f t="shared" ca="1" si="25"/>
+        <f t="shared" ca="1" si="13"/>
         <v>46049</v>
       </c>
       <c r="C41" s="12"/>
@@ -7720,7 +7651,7 @@
       <c r="H41" s="21"/>
       <c r="I41" s="19"/>
       <c r="J41" s="13">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" ca="1" si="11"/>
         <v>46080</v>
       </c>
       <c r="K41" s="12"/>
@@ -7731,7 +7662,7 @@
       <c r="P41" s="21"/>
       <c r="Q41" s="19"/>
       <c r="R41" s="13">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="0"/>
         <v>46108</v>
       </c>
       <c r="S41" s="12"/>
@@ -7742,7 +7673,7 @@
       <c r="X41" s="21"/>
       <c r="Y41" s="19"/>
       <c r="Z41" s="13">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" ca="1" si="1"/>
         <v>46139</v>
       </c>
       <c r="AA41" s="12"/>
@@ -7753,7 +7684,7 @@
       <c r="AF41" s="21"/>
       <c r="AG41" s="19"/>
       <c r="AH41" s="13">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" ca="1" si="2"/>
         <v>46169</v>
       </c>
       <c r="AI41" s="12"/>
@@ -7764,7 +7695,7 @@
       <c r="AN41" s="21"/>
       <c r="AO41" s="19"/>
       <c r="AP41" s="13">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="3"/>
         <v>46200</v>
       </c>
       <c r="AQ41" s="12"/>
@@ -7775,7 +7706,7 @@
       <c r="AV41" s="21"/>
       <c r="AW41" s="19"/>
       <c r="AX41" s="13">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="4"/>
         <v>46230</v>
       </c>
       <c r="AY41" s="12"/>
@@ -7786,7 +7717,7 @@
       <c r="BD41" s="21"/>
       <c r="BE41" s="19"/>
       <c r="BF41" s="13">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" ca="1" si="5"/>
         <v>46261</v>
       </c>
       <c r="BG41" s="12"/>
@@ -7797,7 +7728,7 @@
       <c r="BL41" s="21"/>
       <c r="BM41" s="19"/>
       <c r="BN41" s="13">
-        <f t="shared" ca="1" si="18"/>
+        <f t="shared" ca="1" si="6"/>
         <v>46292</v>
       </c>
       <c r="BO41" s="12"/>
@@ -7808,7 +7739,7 @@
       <c r="BT41" s="21"/>
       <c r="BU41" s="19"/>
       <c r="BV41" s="13">
-        <f t="shared" ca="1" si="19"/>
+        <f t="shared" ca="1" si="7"/>
         <v>46322</v>
       </c>
       <c r="BW41" s="12"/>
@@ -7819,7 +7750,7 @@
       <c r="CB41" s="21"/>
       <c r="CC41" s="19"/>
       <c r="CD41" s="13">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" ca="1" si="8"/>
         <v>46353</v>
       </c>
       <c r="CE41" s="12"/>
@@ -7830,7 +7761,7 @@
       <c r="CJ41" s="21"/>
       <c r="CK41" s="19"/>
       <c r="CL41" s="13">
-        <f t="shared" ca="1" si="21"/>
+        <f t="shared" ca="1" si="9"/>
         <v>46383</v>
       </c>
       <c r="CM41" s="12"/>
@@ -7844,7 +7775,7 @@
     <row r="42" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="1"/>
       <c r="B42" s="13">
-        <f t="shared" ca="1" si="25"/>
+        <f t="shared" ca="1" si="13"/>
         <v>46050</v>
       </c>
       <c r="C42" s="12"/>
@@ -7855,7 +7786,7 @@
       <c r="H42" s="21"/>
       <c r="I42" s="19"/>
       <c r="J42" s="13">
-        <f t="shared" ca="1" si="23"/>
+        <f t="shared" ca="1" si="11"/>
         <v>46081</v>
       </c>
       <c r="K42" s="12"/>
@@ -7866,7 +7797,7 @@
       <c r="P42" s="21"/>
       <c r="Q42" s="19"/>
       <c r="R42" s="13">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="0"/>
         <v>46109</v>
       </c>
       <c r="S42" s="12"/>
@@ -7877,7 +7808,7 @@
       <c r="X42" s="21"/>
       <c r="Y42" s="19"/>
       <c r="Z42" s="13">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" ca="1" si="1"/>
         <v>46140</v>
       </c>
       <c r="AA42" s="12"/>
@@ -7888,7 +7819,7 @@
       <c r="AF42" s="21"/>
       <c r="AG42" s="19"/>
       <c r="AH42" s="13">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" ca="1" si="2"/>
         <v>46170</v>
       </c>
       <c r="AI42" s="12"/>
@@ -7899,7 +7830,7 @@
       <c r="AN42" s="21"/>
       <c r="AO42" s="19"/>
       <c r="AP42" s="13">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="3"/>
         <v>46201</v>
       </c>
       <c r="AQ42" s="12"/>
@@ -7910,7 +7841,7 @@
       <c r="AV42" s="21"/>
       <c r="AW42" s="19"/>
       <c r="AX42" s="13">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="4"/>
         <v>46231</v>
       </c>
       <c r="AY42" s="12"/>
@@ -7921,7 +7852,7 @@
       <c r="BD42" s="21"/>
       <c r="BE42" s="19"/>
       <c r="BF42" s="13">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" ca="1" si="5"/>
         <v>46262</v>
       </c>
       <c r="BG42" s="12"/>
@@ -7932,7 +7863,7 @@
       <c r="BL42" s="21"/>
       <c r="BM42" s="19"/>
       <c r="BN42" s="13">
-        <f t="shared" ca="1" si="18"/>
+        <f t="shared" ca="1" si="6"/>
         <v>46293</v>
       </c>
       <c r="BO42" s="12"/>
@@ -7943,7 +7874,7 @@
       <c r="BT42" s="21"/>
       <c r="BU42" s="19"/>
       <c r="BV42" s="13">
-        <f t="shared" ca="1" si="19"/>
+        <f t="shared" ca="1" si="7"/>
         <v>46323</v>
       </c>
       <c r="BW42" s="12"/>
@@ -7954,7 +7885,7 @@
       <c r="CB42" s="21"/>
       <c r="CC42" s="19"/>
       <c r="CD42" s="13">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" ca="1" si="8"/>
         <v>46354</v>
       </c>
       <c r="CE42" s="12"/>
@@ -7965,7 +7896,7 @@
       <c r="CJ42" s="21"/>
       <c r="CK42" s="19"/>
       <c r="CL42" s="13">
-        <f t="shared" ca="1" si="21"/>
+        <f t="shared" ca="1" si="9"/>
         <v>46384</v>
       </c>
       <c r="CM42" s="12"/>
@@ -7979,7 +7910,7 @@
     <row r="43" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="1"/>
       <c r="B43" s="13">
-        <f t="shared" ca="1" si="25"/>
+        <f t="shared" ca="1" si="13"/>
         <v>46051</v>
       </c>
       <c r="C43" s="12"/>
@@ -7998,7 +7929,7 @@
       <c r="P43" s="19"/>
       <c r="Q43" s="19"/>
       <c r="R43" s="13">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="0"/>
         <v>46110</v>
       </c>
       <c r="S43" s="12"/>
@@ -8009,7 +7940,7 @@
       <c r="X43" s="21"/>
       <c r="Y43" s="19"/>
       <c r="Z43" s="13">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" ca="1" si="1"/>
         <v>46141</v>
       </c>
       <c r="AA43" s="12"/>
@@ -8020,7 +7951,7 @@
       <c r="AF43" s="21"/>
       <c r="AG43" s="19"/>
       <c r="AH43" s="13">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" ca="1" si="2"/>
         <v>46171</v>
       </c>
       <c r="AI43" s="12"/>
@@ -8031,7 +7962,7 @@
       <c r="AN43" s="21"/>
       <c r="AO43" s="19"/>
       <c r="AP43" s="13">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="3"/>
         <v>46202</v>
       </c>
       <c r="AQ43" s="12"/>
@@ -8042,7 +7973,7 @@
       <c r="AV43" s="21"/>
       <c r="AW43" s="19"/>
       <c r="AX43" s="13">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="4"/>
         <v>46232</v>
       </c>
       <c r="AY43" s="12"/>
@@ -8053,7 +7984,7 @@
       <c r="BD43" s="21"/>
       <c r="BE43" s="19"/>
       <c r="BF43" s="13">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" ca="1" si="5"/>
         <v>46263</v>
       </c>
       <c r="BG43" s="12"/>
@@ -8064,7 +7995,7 @@
       <c r="BL43" s="21"/>
       <c r="BM43" s="19"/>
       <c r="BN43" s="13">
-        <f t="shared" ca="1" si="18"/>
+        <f t="shared" ca="1" si="6"/>
         <v>46294</v>
       </c>
       <c r="BO43" s="12" t="s">
@@ -8077,7 +8008,7 @@
       <c r="BT43" s="21"/>
       <c r="BU43" s="19"/>
       <c r="BV43" s="13">
-        <f t="shared" ca="1" si="19"/>
+        <f t="shared" ca="1" si="7"/>
         <v>46324</v>
       </c>
       <c r="BW43" s="12"/>
@@ -8088,7 +8019,7 @@
       <c r="CB43" s="21"/>
       <c r="CC43" s="19"/>
       <c r="CD43" s="13">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" ca="1" si="8"/>
         <v>46355</v>
       </c>
       <c r="CE43" s="12"/>
@@ -8099,7 +8030,7 @@
       <c r="CJ43" s="21"/>
       <c r="CK43" s="19"/>
       <c r="CL43" s="13">
-        <f t="shared" ca="1" si="21"/>
+        <f t="shared" ca="1" si="9"/>
         <v>46385</v>
       </c>
       <c r="CM43" s="12"/>
@@ -8113,7 +8044,7 @@
     <row r="44" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="1"/>
       <c r="B44" s="13">
-        <f t="shared" ca="1" si="25"/>
+        <f t="shared" ca="1" si="13"/>
         <v>46052</v>
       </c>
       <c r="C44" s="12"/>
@@ -8132,7 +8063,7 @@
       <c r="P44" s="19"/>
       <c r="Q44" s="19"/>
       <c r="R44" s="13">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="0"/>
         <v>46111</v>
       </c>
       <c r="S44" s="12"/>
@@ -8143,7 +8074,7 @@
       <c r="X44" s="21"/>
       <c r="Y44" s="19"/>
       <c r="Z44" s="13">
-        <f t="shared" ca="1" si="13"/>
+        <f t="shared" ca="1" si="1"/>
         <v>46142</v>
       </c>
       <c r="AA44" s="12"/>
@@ -8154,7 +8085,7 @@
       <c r="AF44" s="21"/>
       <c r="AG44" s="19"/>
       <c r="AH44" s="13">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" ca="1" si="2"/>
         <v>46172</v>
       </c>
       <c r="AI44" s="12"/>
@@ -8165,7 +8096,7 @@
       <c r="AN44" s="21"/>
       <c r="AO44" s="19"/>
       <c r="AP44" s="13">
-        <f t="shared" ca="1" si="15"/>
+        <f t="shared" ca="1" si="3"/>
         <v>46203</v>
       </c>
       <c r="AQ44" s="12"/>
@@ -8176,7 +8107,7 @@
       <c r="AV44" s="21"/>
       <c r="AW44" s="19"/>
       <c r="AX44" s="13">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="4"/>
         <v>46233</v>
       </c>
       <c r="AY44" s="12"/>
@@ -8187,7 +8118,7 @@
       <c r="BD44" s="21"/>
       <c r="BE44" s="19"/>
       <c r="BF44" s="13">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" ca="1" si="5"/>
         <v>46264</v>
       </c>
       <c r="BG44" s="12"/>
@@ -8198,7 +8129,7 @@
       <c r="BL44" s="21"/>
       <c r="BM44" s="19"/>
       <c r="BN44" s="13">
-        <f t="shared" ca="1" si="18"/>
+        <f t="shared" ca="1" si="6"/>
         <v>46295</v>
       </c>
       <c r="BO44" s="12"/>
@@ -8209,7 +8140,7 @@
       <c r="BT44" s="21"/>
       <c r="BU44" s="19"/>
       <c r="BV44" s="13">
-        <f t="shared" ca="1" si="19"/>
+        <f t="shared" ca="1" si="7"/>
         <v>46325</v>
       </c>
       <c r="BW44" s="12"/>
@@ -8220,7 +8151,7 @@
       <c r="CB44" s="21"/>
       <c r="CC44" s="19"/>
       <c r="CD44" s="13">
-        <f t="shared" ca="1" si="20"/>
+        <f t="shared" ca="1" si="8"/>
         <v>46356</v>
       </c>
       <c r="CE44" s="12"/>
@@ -8231,7 +8162,7 @@
       <c r="CJ44" s="21"/>
       <c r="CK44" s="19"/>
       <c r="CL44" s="13">
-        <f t="shared" ca="1" si="21"/>
+        <f t="shared" ca="1" si="9"/>
         <v>46386</v>
       </c>
       <c r="CM44" s="12"/>
@@ -8245,7 +8176,7 @@
     <row r="45" spans="1:97" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="1"/>
       <c r="B45" s="13">
-        <f t="shared" ca="1" si="25"/>
+        <f t="shared" ca="1" si="13"/>
         <v>46053</v>
       </c>
       <c r="C45" s="12"/>
@@ -8264,7 +8195,7 @@
       <c r="P45" s="19"/>
       <c r="Q45" s="19"/>
       <c r="R45" s="13">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="0"/>
         <v>46112</v>
       </c>
       <c r="S45" s="12"/>
@@ -8283,7 +8214,7 @@
       <c r="AF45" s="19"/>
       <c r="AG45" s="19"/>
       <c r="AH45" s="13">
-        <f t="shared" ca="1" si="14"/>
+        <f t="shared" ca="1" si="2"/>
         <v>46173</v>
       </c>
       <c r="AI45" s="12"/>
@@ -8302,7 +8233,7 @@
       <c r="AV45" s="19"/>
       <c r="AW45" s="19"/>
       <c r="AX45" s="13">
-        <f t="shared" ca="1" si="16"/>
+        <f t="shared" ca="1" si="4"/>
         <v>46234</v>
       </c>
       <c r="AY45" s="12"/>
@@ -8313,7 +8244,7 @@
       <c r="BD45" s="21"/>
       <c r="BE45" s="19"/>
       <c r="BF45" s="13">
-        <f t="shared" ca="1" si="17"/>
+        <f t="shared" ca="1" si="5"/>
         <v>46265</v>
       </c>
       <c r="BG45" s="12"/>
@@ -8332,7 +8263,7 @@
       <c r="BT45" s="19"/>
       <c r="BU45" s="19"/>
       <c r="BV45" s="13">
-        <f t="shared" ca="1" si="19"/>
+        <f t="shared" ca="1" si="7"/>
         <v>46326</v>
       </c>
       <c r="BW45" s="12"/>
@@ -8351,7 +8282,7 @@
       <c r="CJ45" s="22"/>
       <c r="CK45" s="19"/>
       <c r="CL45" s="13">
-        <f t="shared" ca="1" si="21"/>
+        <f t="shared" ca="1" si="9"/>
         <v>46387</v>
       </c>
       <c r="CM45" s="12"/>
@@ -8775,7 +8706,7 @@
       </c>
       <c r="B2" s="24">
         <f ca="1">NOW()</f>
-        <v>46226.526188541669</v>
+        <v>46233.610213888889</v>
       </c>
     </row>
   </sheetData>

</xml_diff>